<commit_message>
docs(scrum): actualizar burndown chart y actas del sprint 2
</commit_message>
<xml_diff>
--- a/scrum/burndown/PubTube_Burndown_B_S2.xlsx
+++ b/scrum/burndown/PubTube_Burndown_B_S2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccien\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccien\Documents\github\PubTube-Modulo2\scrum\burndown\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A966213C-C4B2-4133-B9F9-6A4128088A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6AC42B-5358-4EDA-B56E-8FAD48D4BE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="⚙ Configuración" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="🔄 Retrospectiva" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="178">
   <si>
     <t>🏃  Configuración del Sprint</t>
   </si>
@@ -198,12 +197,6 @@
   </si>
   <si>
     <t>Dead-letter queue observable y reprocesable</t>
-  </si>
-  <si>
-    <t>US-B4</t>
-  </si>
-  <si>
-    <t>Idempotencia de consumidores</t>
   </si>
   <si>
     <t>To Do</t>
@@ -561,42 +554,18 @@
     <t>🔄  Retrospectiva del Sprint</t>
   </si>
   <si>
-    <t>Retrospectiva del Sprint 1</t>
-  </si>
-  <si>
     <t>✅  KEEP — Lo que funcionó bien</t>
   </si>
   <si>
     <t xml:space="preserve">  •  Todas las funciones solicitadas por las historias de usuario fueron hechas dentro del tiempo establecido</t>
   </si>
   <si>
-    <t xml:space="preserve">  •  la division de historias de usuario para el sprint 1 resulto ser correcta y efectiva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  •  ...</t>
-  </si>
-  <si>
     <t>❌  DROP — Lo que hay que dejar de hacer</t>
   </si>
   <si>
-    <t xml:space="preserve">  •  Una buena parte de la carga de trabajo se terminó desplazando hacia fechas criticas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • no hubo una planificacion sobre como abordar la presentación del sprint 1</t>
-  </si>
-  <si>
     <t>🚀  TRY — Lo que queremos intentar</t>
   </si>
   <si>
-    <t xml:space="preserve">  •  redistribuir de mejor manera los SPs de ls historias de usuario a lo largo del tiempo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  •  implementar un plan de presentación de sprint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  •  Continuar en base a la guia de las historias de usuario refinadas</t>
-  </si>
-  <si>
     <t>📌  Acciones Concretas para el Próximo Sprint</t>
   </si>
   <si>
@@ -628,6 +597,48 @@
   </si>
   <si>
     <t>equipo completo</t>
+  </si>
+  <si>
+    <t>US-B4a</t>
+  </si>
+  <si>
+    <t>Persistencia y control de concurrencia de idempotencia</t>
+  </si>
+  <si>
+    <t>Wrapper reutilizable, consumidor de prueba y documentación</t>
+  </si>
+  <si>
+    <t>US-B4b</t>
+  </si>
+  <si>
+    <t>Adolfo</t>
+  </si>
+  <si>
+    <t>Adolfo - Carlos</t>
+  </si>
+  <si>
+    <t>Adolfo - Carlos - Eduardo</t>
+  </si>
+  <si>
+    <t>3 y 4</t>
+  </si>
+  <si>
+    <t>Retrospectiva del Sprint 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  •  la mayoria de los SP se realizaron en las ultimas sesiones del sprint, lo que ajustó el tiempo para probar el gateway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  •  mejorar la comunicación/coordinación con los demás módulos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  •  hubo unas sesiones de retraso para hacer el planning por lo que no hubo mucho avance, ya que habia que reajustar la documentación del sprint 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  •  Hubo mayor cantidad de trabajo, lo cúal vino bien ya que este sprint era más grande que el anterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  •  redistribuir de mejor manera los SPs de las historias de usuario a lo largo del tiempo</t>
   </si>
 </sst>
 </file>
@@ -643,7 +654,7 @@
     <numFmt numFmtId="169" formatCode="dd/mm"/>
     <numFmt numFmtId="170" formatCode="d/m"/>
   </numFmts>
-  <fonts count="34" x14ac:knownFonts="1">
+  <fonts count="39" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -839,6 +850,38 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1A2E4A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF64748B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF64748B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1A2E4A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="15">
@@ -1051,7 +1094,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1240,39 +1283,29 @@
     <xf numFmtId="170" fontId="32" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1286,10 +1319,37 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1298,53 +1358,17 @@
     <xf numFmtId="0" fontId="30" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6600"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4" tint="0.79998168889431442"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="8" tint="0.79998168889431442"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <font>
         <color theme="9" tint="0.59996337778862885"/>
@@ -1367,11 +1391,11 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="4" tint="0.79998168889431442"/>
+        <color theme="8" tint="0.79998168889431442"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FF0070C0"/>
+          <bgColor theme="8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1382,6 +1406,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4" tint="0.79998168889431442"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2063,11 +2097,6 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="8064A2">
-                <a:alpha val="30000"/>
-              </a:srgbClr>
-            </a:solidFill>
             <a:ln w="47625" cmpd="sng">
               <a:noFill/>
               <a:prstDash val="solid"/>
@@ -3037,11 +3066,6 @@
             <c:v>SP por sprint</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="8064A2">
-                <a:alpha val="30000"/>
-              </a:srgbClr>
-            </a:solidFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -3909,58 +3933,58 @@
                   <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>49</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>49</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3995,11 +4019,6 @@
             <c:v>SP por sprint</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="8064A2">
-                <a:alpha val="30000"/>
-              </a:srgbClr>
-            </a:solidFill>
             <a:ln w="47625" cmpd="sng">
               <a:noFill/>
               <a:prstDash val="solid"/>
@@ -4115,7 +4134,7 @@
                   <c:v>63</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>42</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>13</c:v>
@@ -4672,58 +4691,58 @@
                   <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>27</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>27</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4978,11 +4997,6 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="8064A2">
-                <a:alpha val="30000"/>
-              </a:srgbClr>
-            </a:solidFill>
             <a:ln w="47625" cmpd="sng">
               <a:noFill/>
               <a:prstDash val="solid"/>
@@ -5373,9 +5387,9 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>488156</xdr:colOff>
+      <xdr:row>2</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5791200" cy="3209925"/>
@@ -5404,10 +5418,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>488156</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>73819</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5791200" cy="3209925"/>
     <xdr:graphicFrame macro="">
@@ -5649,22 +5663,22 @@
       <c r="B1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="68"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="73"/>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="68"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="73"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="73" t="s">
+      <c r="B3" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="68"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="73"/>
     </row>
     <row r="4" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
@@ -5725,7 +5739,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="2">
-        <f>'📋 Sprint Backlog'!F27</f>
+        <f>'📋 Sprint Backlog'!F28</f>
         <v>76</v>
       </c>
       <c r="D10" s="3"/>
@@ -5749,75 +5763,75 @@
       <c r="D12" s="3"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="73" t="s">
+      <c r="B13" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="67"/>
-      <c r="D13" s="68"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="73"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="78" t="s">
+      <c r="B14" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="67"/>
-      <c r="D14" s="68"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="73"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="78" t="s">
+      <c r="B15" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="67"/>
-      <c r="D15" s="68"/>
+      <c r="C15" s="72"/>
+      <c r="D15" s="73"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="78" t="s">
+      <c r="B16" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="67"/>
-      <c r="D16" s="68"/>
+      <c r="C16" s="72"/>
+      <c r="D16" s="73"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="78" t="s">
+      <c r="B17" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="67"/>
-      <c r="D17" s="68"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="73"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="78" t="s">
+      <c r="B18" s="75" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="67"/>
-      <c r="D18" s="68"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="73"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="74" t="s">
+      <c r="B19" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="67"/>
-      <c r="D19" s="68"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="73"/>
     </row>
     <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="79" t="s">
+      <c r="B20" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="80"/>
-      <c r="D20" s="81"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="79"/>
     </row>
     <row r="21" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="82"/>
-      <c r="C21" s="83"/>
-      <c r="D21" s="84"/>
+      <c r="B21" s="80"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="82"/>
     </row>
     <row r="22" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="82"/>
-      <c r="C22" s="83"/>
-      <c r="D22" s="84"/>
+      <c r="B22" s="80"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="82"/>
     </row>
     <row r="23" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="85"/>
-      <c r="C23" s="86"/>
-      <c r="D23" s="87"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="84"/>
+      <c r="D23" s="85"/>
     </row>
     <row r="24" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6817,7 +6831,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B1:K1007"/>
+  <dimension ref="B1:K1008"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -6836,25 +6850,25 @@
       <c r="B1" s="71" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="68"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="73"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="68"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="73"/>
     </row>
     <row r="3" spans="2:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
@@ -7039,66 +7053,74 @@
       </c>
     </row>
     <row r="10" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="10" t="s">
-        <v>52</v>
+      <c r="B10" s="68" t="s">
+        <v>164</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>53</v>
+        <v>165</v>
       </c>
       <c r="D10" s="12">
         <v>2</v>
       </c>
-      <c r="E10" s="13"/>
+      <c r="E10" s="69" t="s">
+        <v>39</v>
+      </c>
       <c r="F10" s="14">
-        <v>5</v>
-      </c>
-      <c r="G10" s="15"/>
+        <v>3</v>
+      </c>
+      <c r="G10" s="15">
+        <v>3</v>
+      </c>
       <c r="H10" s="16" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="I10" s="17" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="10" t="s">
-        <v>55</v>
+      <c r="B11" s="68" t="s">
+        <v>167</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>56</v>
+        <v>166</v>
       </c>
       <c r="D11" s="12">
-        <v>3</v>
-      </c>
-      <c r="E11" s="13"/>
+        <v>2</v>
+      </c>
+      <c r="E11" s="69" t="s">
+        <v>39</v>
+      </c>
       <c r="F11" s="14">
-        <v>5</v>
-      </c>
-      <c r="G11" s="15"/>
+        <v>2</v>
+      </c>
+      <c r="G11" s="15">
+        <v>2</v>
+      </c>
       <c r="H11" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="I11" s="18" t="s">
-        <v>46</v>
+        <v>35</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D12" s="12">
         <v>3</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G12" s="15"/>
       <c r="H12" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I12" s="18" t="s">
         <v>46</v>
@@ -7106,47 +7128,43 @@
     </row>
     <row r="13" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="10" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D13" s="12">
-        <v>2</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>61</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="E13" s="13"/>
       <c r="F13" s="14">
         <v>3</v>
       </c>
-      <c r="G13" s="15">
-        <v>3</v>
-      </c>
+      <c r="G13" s="15"/>
       <c r="H13" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="I13" s="17" t="s">
-        <v>36</v>
+        <v>52</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="10" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D14" s="12">
         <v>2</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="F14" s="14">
         <v>3</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="15">
         <v>3</v>
       </c>
       <c r="H14" s="16" t="s">
@@ -7158,58 +7176,62 @@
     </row>
     <row r="15" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D15" s="12">
+        <v>2</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="14">
         <v>3</v>
       </c>
-      <c r="E15" s="13"/>
-      <c r="F15" s="14">
-        <v>5</v>
-      </c>
-      <c r="G15" s="15"/>
+      <c r="G15" s="14">
+        <v>3</v>
+      </c>
       <c r="H15" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="I15" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="K15" s="93"/>
+        <v>35</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="16" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D16" s="12">
         <v>3</v>
       </c>
       <c r="E16" s="13"/>
       <c r="F16" s="14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I16" s="18" t="s">
         <v>46</v>
       </c>
+      <c r="K16" s="66"/>
     </row>
     <row r="17" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="10" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D17" s="12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" s="13"/>
       <c r="F17" s="14">
@@ -7217,87 +7239,87 @@
       </c>
       <c r="G17" s="15"/>
       <c r="H17" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I17" s="18" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="10" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D18" s="12">
-        <v>4</v>
+        <v>67</v>
+      </c>
+      <c r="D18" s="70" t="s">
+        <v>171</v>
       </c>
       <c r="E18" s="13"/>
       <c r="F18" s="14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G18" s="15"/>
       <c r="H18" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I18" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="D19" s="12">
-        <v>4</v>
+        <v>70</v>
+      </c>
+      <c r="D19" s="70" t="s">
+        <v>171</v>
       </c>
       <c r="E19" s="13"/>
       <c r="F19" s="14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G19" s="15"/>
       <c r="H19" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I19" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="10" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="12">
-        <v>4</v>
+        <v>72</v>
+      </c>
+      <c r="D20" s="70" t="s">
+        <v>171</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G20" s="15"/>
       <c r="H20" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I20" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" s="12">
-        <v>2</v>
+        <v>74</v>
+      </c>
+      <c r="D21" s="70" t="s">
+        <v>171</v>
       </c>
       <c r="E21" s="13"/>
       <c r="F21" s="14">
@@ -7305,29 +7327,33 @@
       </c>
       <c r="G21" s="15"/>
       <c r="H21" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I21" s="18" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D22" s="12">
         <v>2</v>
       </c>
-      <c r="E22" s="13"/>
+      <c r="E22" s="69" t="s">
+        <v>168</v>
+      </c>
       <c r="F22" s="14">
-        <v>2</v>
-      </c>
-      <c r="G22" s="15"/>
+        <v>3</v>
+      </c>
+      <c r="G22" s="15">
+        <v>3</v>
+      </c>
       <c r="H22" s="16" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="I22" s="18" t="s">
         <v>36</v>
@@ -7335,21 +7361,25 @@
     </row>
     <row r="23" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D23" s="12">
         <v>2</v>
       </c>
-      <c r="E23" s="13"/>
+      <c r="E23" s="69" t="s">
+        <v>169</v>
+      </c>
       <c r="F23" s="14">
         <v>2</v>
       </c>
-      <c r="G23" s="15"/>
+      <c r="G23" s="15">
+        <v>2</v>
+      </c>
       <c r="H23" s="16" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="I23" s="18" t="s">
         <v>36</v>
@@ -7357,21 +7387,25 @@
     </row>
     <row r="24" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D24" s="12">
         <v>2</v>
       </c>
-      <c r="E24" s="13"/>
+      <c r="E24" s="69" t="s">
+        <v>168</v>
+      </c>
       <c r="F24" s="14">
-        <v>3</v>
-      </c>
-      <c r="G24" s="15"/>
+        <v>2</v>
+      </c>
+      <c r="G24" s="15">
+        <v>2</v>
+      </c>
       <c r="H24" s="16" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="I24" s="18" t="s">
         <v>36</v>
@@ -7379,73 +7413,96 @@
     </row>
     <row r="25" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D25" s="12">
+        <v>2</v>
+      </c>
+      <c r="E25" s="69" t="s">
+        <v>170</v>
+      </c>
+      <c r="F25" s="14">
         <v>3</v>
       </c>
-      <c r="E25" s="13"/>
-      <c r="F25" s="14">
-        <v>2</v>
-      </c>
-      <c r="G25" s="15"/>
+      <c r="G25" s="15">
+        <v>3</v>
+      </c>
       <c r="H25" s="16" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="I25" s="18" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="10" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D26" s="12">
         <v>3</v>
       </c>
       <c r="E26" s="13"/>
       <c r="F26" s="14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G26" s="15"/>
       <c r="H26" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I26" s="18" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="2:9" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B27" s="88" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="67"/>
-      <c r="D27" s="67"/>
-      <c r="E27" s="68"/>
-      <c r="F27" s="19">
-        <f t="shared" ref="F27:G27" si="0">SUM(F4:F26)</f>
+    <row r="27" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D27" s="12">
+        <v>3</v>
+      </c>
+      <c r="E27" s="13"/>
+      <c r="F27" s="14">
+        <v>3</v>
+      </c>
+      <c r="G27" s="15"/>
+      <c r="H27" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="I27" s="18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="B28" s="87" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" s="72"/>
+      <c r="D28" s="72"/>
+      <c r="E28" s="73"/>
+      <c r="F28" s="19">
+        <f t="shared" ref="F28:G28" si="0">SUM(F4:F27)</f>
         <v>76</v>
       </c>
-      <c r="G27" s="20">
+      <c r="G28" s="20">
         <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="H27" s="21">
-        <f>IFERROR(G27/F27,0)</f>
-        <v>0.35526315789473684</v>
-      </c>
-      <c r="I27" s="22"/>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D28" s="23"/>
-    </row>
-    <row r="29" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="H28" s="21">
+        <f>IFERROR(G28/F28,0)</f>
+        <v>0.55263157894736847</v>
+      </c>
+      <c r="I28" s="22"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D29" s="23"/>
     </row>
     <row r="30" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10381,42 +10438,46 @@
     </row>
     <row r="1007" spans="4:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1007" s="23"/>
+    </row>
+    <row r="1008" spans="4:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D1008" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
   </mergeCells>
-  <conditionalFormatting sqref="H4:H26">
-    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="To Do">
+  <phoneticPr fontId="37" type="noConversion"/>
+  <conditionalFormatting sqref="H4:H27">
+    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="Done">
+      <formula>NOT(ISERROR(SEARCH("Done",H4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="To Do">
       <formula>NOT(ISERROR(SEARCH("To Do",H4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH("Done",H4)))</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4:I27">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Baja">
+      <formula>NOT(ISERROR(SEARCH("Baja",I4)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I26">
-    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="Alta">
-      <formula>NOT(ISERROR(SEARCH("Alta",I4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Medio">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Medio">
       <formula>NOT(ISERROR(SEARCH("Medio",I4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Baja">
-      <formula>NOT(ISERROR(SEARCH("Baja",I4)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Alta">
+      <formula>NOT(ISERROR(SEARCH("Alta",I4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H4:H26" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H4:H27" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Done,To Do"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I4:I26" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I4:I27" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Alta,Medio,Baja"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10429,8 +10490,7 @@
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="4" width="14" customWidth="1"/>
     <col min="5" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="12.85546875" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
@@ -10440,59 +10500,59 @@
   <sheetData>
     <row r="1" spans="2:13" ht="21" x14ac:dyDescent="0.25">
       <c r="B1" s="71" t="s">
-        <v>90</v>
-      </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="68"/>
+        <v>88</v>
+      </c>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="73"/>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="72" t="s">
-        <v>91</v>
-      </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="68"/>
+      <c r="B2" s="74" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="73"/>
     </row>
     <row r="3" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="F3" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="H3" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="I3" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="J3" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="G3" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="H3" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="I3" s="33" t="s">
+      <c r="K3" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="J3" s="33" t="s">
+      <c r="L3" s="34" t="s">
         <v>101</v>
-      </c>
-      <c r="K3" s="33" t="s">
-        <v>102</v>
-      </c>
-      <c r="L3" s="34" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="4" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10558,7 +10618,7 @@
         <f>IF($B5&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B5 - 1) / 24)</f>
         <v>3.1666666666666665</v>
       </c>
-      <c r="K5" s="94"/>
+      <c r="K5" s="67"/>
       <c r="L5" s="39"/>
     </row>
     <row r="6" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10592,7 +10652,7 @@
         <f>IF($B6&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B6 - 1) / 24)</f>
         <v>6.333333333333333</v>
       </c>
-      <c r="K6" s="94"/>
+      <c r="K6" s="67"/>
       <c r="L6" s="39"/>
     </row>
     <row r="7" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10626,10 +10686,10 @@
         <f>IF($B7&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B7 - 1) / 24)</f>
         <v>9.5</v>
       </c>
-      <c r="K7" s="94"/>
+      <c r="K7" s="67"/>
       <c r="L7" s="39"/>
       <c r="M7" s="31" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10660,10 +10720,10 @@
         <f>IF($B8&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B8 - 1) / 24)</f>
         <v>12.666666666666666</v>
       </c>
-      <c r="K8" s="94"/>
+      <c r="K8" s="67"/>
       <c r="L8" s="39"/>
       <c r="M8" s="40" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10704,7 +10764,7 @@
         <v>63</v>
       </c>
       <c r="M9" s="40" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11426,7 +11486,7 @@
     <row r="35" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H37" s="94"/>
+      <c r="H37" s="67"/>
     </row>
     <row r="38" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12416,67 +12476,68 @@
     <col min="3" max="4" width="14" customWidth="1"/>
     <col min="5" max="6" width="16" customWidth="1"/>
     <col min="7" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="12.85546875" hidden="1" customWidth="1"/>
-    <col min="11" max="12" width="9.7109375" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="9" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="7.42578125" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="18.5703125" hidden="1" customWidth="1"/>
     <col min="13" max="31" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="21" x14ac:dyDescent="0.25">
       <c r="B1" s="71" t="s">
-        <v>90</v>
-      </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="68"/>
+        <v>88</v>
+      </c>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="73"/>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="72" t="s">
-        <v>91</v>
-      </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="68"/>
+      <c r="B2" s="74" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="73"/>
     </row>
     <row r="3" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="F3" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="H3" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="I3" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="J3" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="G3" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="H3" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="I3" s="33" t="s">
+      <c r="K3" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="J3" s="33" t="s">
+      <c r="L3" s="34" t="s">
         <v>101</v>
-      </c>
-      <c r="K3" s="33" t="s">
-        <v>102</v>
-      </c>
-      <c r="L3" s="34" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="4" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12612,9 +12673,7 @@
       </c>
       <c r="K7" s="39"/>
       <c r="L7" s="39"/>
-      <c r="M7" s="31" t="s">
-        <v>98</v>
-      </c>
+      <c r="M7" s="31"/>
     </row>
     <row r="8" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="28">
@@ -12647,7 +12706,7 @@
       <c r="K8" s="39"/>
       <c r="L8" s="39"/>
       <c r="M8" s="40" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12688,7 +12747,7 @@
         <v>63</v>
       </c>
       <c r="M9" s="40" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12836,14 +12895,17 @@
         <f>IF($B14&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B14) / 24)</f>
         <v>44.333333333333336</v>
       </c>
-      <c r="F14" s="15"/>
+      <c r="F14" s="15">
+        <f>2+3+3</f>
+        <v>8</v>
+      </c>
       <c r="G14" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="H14" s="36">
         <f>'⚙ Configuración'!$C$10-G14</f>
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="I14" s="37"/>
       <c r="J14" s="38">
@@ -12868,14 +12930,17 @@
         <f>IF($B15&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B15) / 24)</f>
         <v>41.166666666666664</v>
       </c>
-      <c r="F15" s="15"/>
+      <c r="F15" s="15">
+        <f>3+2+2</f>
+        <v>7</v>
+      </c>
       <c r="G15" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H15" s="36">
         <f>'⚙ Configuración'!$C$10-G15</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I15" s="37">
         <f>'⚙ Configuración'!$C$10</f>
@@ -12889,7 +12954,8 @@
         <v>42</v>
       </c>
       <c r="L15" s="39">
-        <v>42</v>
+        <f>76-42</f>
+        <v>34</v>
       </c>
       <c r="M15" s="31"/>
     </row>
@@ -12910,11 +12976,11 @@
       <c r="F16" s="15"/>
       <c r="G16" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H16" s="36">
         <f>'⚙ Configuración'!$C$10-G16</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I16" s="37"/>
       <c r="J16" s="38">
@@ -12941,11 +13007,11 @@
       <c r="F17" s="15"/>
       <c r="G17" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H17" s="36">
         <f>'⚙ Configuración'!$C$10-G17</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I17" s="37"/>
       <c r="J17" s="38">
@@ -12972,11 +13038,11 @@
       <c r="F18" s="15"/>
       <c r="G18" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H18" s="36">
         <f>'⚙ Configuración'!$C$10-G18</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I18" s="37"/>
       <c r="J18" s="38">
@@ -13003,11 +13069,11 @@
       <c r="F19" s="15"/>
       <c r="G19" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H19" s="36">
         <f>'⚙ Configuración'!$C$10-G19</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I19" s="37"/>
       <c r="J19" s="38">
@@ -13034,11 +13100,11 @@
       <c r="F20" s="15"/>
       <c r="G20" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H20" s="36">
         <f>'⚙ Configuración'!$C$10-G20</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I20" s="37"/>
       <c r="J20" s="38">
@@ -13065,11 +13131,11 @@
       <c r="F21" s="15"/>
       <c r="G21" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H21" s="36">
         <f>'⚙ Configuración'!$C$10-G21</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I21" s="37">
         <f>'⚙ Configuración'!$C$10</f>
@@ -13083,6 +13149,7 @@
         <v>63</v>
       </c>
       <c r="L21" s="23">
+        <f>76-63</f>
         <v>13</v>
       </c>
     </row>
@@ -13103,11 +13170,11 @@
       <c r="F22" s="15"/>
       <c r="G22" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H22" s="36">
         <f>'⚙ Configuración'!$C$10-G22</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I22" s="37"/>
       <c r="J22" s="38">
@@ -13134,11 +13201,11 @@
       <c r="F23" s="15"/>
       <c r="G23" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H23" s="36">
         <f>'⚙ Configuración'!$C$10-G23</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I23" s="37"/>
       <c r="J23" s="38">
@@ -13165,11 +13232,11 @@
       <c r="F24" s="15"/>
       <c r="G24" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H24" s="36">
         <f>'⚙ Configuración'!$C$10-G24</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I24" s="37"/>
       <c r="J24" s="38">
@@ -13196,11 +13263,11 @@
       <c r="F25" s="15"/>
       <c r="G25" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H25" s="36">
         <f>'⚙ Configuración'!$C$10-G25</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I25" s="37"/>
       <c r="J25" s="38">
@@ -13227,11 +13294,11 @@
       <c r="F26" s="15"/>
       <c r="G26" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H26" s="36">
         <f>'⚙ Configuración'!$C$10-G26</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I26" s="37"/>
       <c r="J26" s="38">
@@ -13258,11 +13325,11 @@
       <c r="F27" s="15"/>
       <c r="G27" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H27" s="36">
         <f>'⚙ Configuración'!$C$10-G27</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I27" s="37"/>
       <c r="J27" s="38">
@@ -13289,11 +13356,11 @@
       <c r="F28" s="15"/>
       <c r="G28" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H28" s="36">
         <f>'⚙ Configuración'!$C$10-G28</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I28" s="37">
         <f>'⚙ Configuración'!$C$10</f>
@@ -13328,11 +13395,11 @@
       <c r="F29" s="15"/>
       <c r="G29" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H29" s="36">
         <f>'⚙ Configuración'!$C$10-G29</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I29" s="37"/>
       <c r="J29" s="38">
@@ -13359,11 +13426,11 @@
       <c r="F30" s="15"/>
       <c r="G30" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H30" s="36">
         <f>'⚙ Configuración'!$C$10-G30</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I30" s="37"/>
       <c r="J30" s="38">
@@ -13390,11 +13457,11 @@
       <c r="F31" s="15"/>
       <c r="G31" s="30">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H31" s="36">
         <f>'⚙ Configuración'!$C$10-G31</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I31" s="37">
         <f>'⚙ Configuración'!$C$10</f>
@@ -13437,7 +13504,7 @@
       <c r="C37" s="23"/>
       <c r="D37" s="23"/>
       <c r="E37" s="23"/>
-      <c r="H37" s="94"/>
+      <c r="H37" s="67"/>
     </row>
     <row r="38" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -14424,7 +14491,7 @@
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="36.7109375" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="56.140625" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="3" customWidth="1"/>
@@ -14433,124 +14500,123 @@
   <sheetData>
     <row r="1" spans="2:5" ht="21" x14ac:dyDescent="0.25">
       <c r="B1" s="71" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="73"/>
+    </row>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="74" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="73"/>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="86" t="s">
         <v>105</v>
       </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="68"/>
-    </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="72" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="68"/>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="73" t="s">
-        <v>107</v>
-      </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="68"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="73"/>
     </row>
     <row r="4" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="41" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C4" s="42">
-        <f>'📋 Sprint Backlog'!F27</f>
+        <f>'📋 Sprint Backlog'!F28</f>
         <v>76</v>
       </c>
       <c r="D4" s="43" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E4" s="44"/>
     </row>
     <row r="5" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C5" s="42">
-        <f>'📋 Sprint Backlog'!G27</f>
-        <v>27</v>
+        <f>'📋 Sprint Backlog'!G28</f>
+        <v>42</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E5" s="45"/>
     </row>
     <row r="6" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="41" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C6" s="42">
-        <f>'📋 Sprint Backlog'!F27-'📋 Sprint Backlog'!G27</f>
-        <v>49</v>
+        <f>'📋 Sprint Backlog'!F28-'📋 Sprint Backlog'!G28</f>
+        <v>34</v>
       </c>
       <c r="D6" s="43" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E6" s="44"/>
     </row>
     <row r="7" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C7" s="46">
-        <f>IFERROR('📋 Sprint Backlog'!G27/'📋 Sprint Backlog'!F27,0)</f>
-        <v>0.35526315789473684</v>
+        <f>IFERROR('📋 Sprint Backlog'!G28/'📋 Sprint Backlog'!F28,0)</f>
+        <v>0.55263157894736847</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E7" s="45"/>
     </row>
     <row r="8" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="41" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C8" s="42">
-        <f>COUNTIF('📋 Sprint Backlog'!H4:H26,"Done")</f>
-        <v>8</v>
+        <f>COUNTIF('📋 Sprint Backlog'!H4:H27,"Done")</f>
+        <v>14</v>
       </c>
       <c r="D8" s="43" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E8" s="44"/>
     </row>
     <row r="9" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="42">
+        <f>COUNTIF('📋 Sprint Backlog'!H4:H27,"To Do")</f>
+        <v>10</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E9" s="45"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="76" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="42">
-        <f>COUNTIF('📋 Sprint Backlog'!H4:H26,"To Do")</f>
-        <v>15</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E9" s="45"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="74" t="s">
-        <v>120</v>
-      </c>
-      <c r="C10" s="67"/>
-      <c r="D10" s="67"/>
-      <c r="E10" s="68"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="73"/>
     </row>
     <row r="11" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C11" s="42">
-        <f>'📋 Sprint Backlog'!G27</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E11" s="45"/>
     </row>
@@ -14563,168 +14629,167 @@
         <v>16</v>
       </c>
       <c r="D12" s="43" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E12" s="44"/>
     </row>
     <row r="13" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C13" s="47">
-        <f>'📋 Sprint Backlog'!G27-'⚙ Configuración'!C11</f>
-        <v>11</v>
+        <f>C11-'⚙ Configuración'!C11</f>
+        <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E13" s="45"/>
     </row>
     <row r="14" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="41" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C14" s="48">
-        <f>IFERROR('📋 Sprint Backlog'!G27/'⚙ Configuración'!C12,0)</f>
-        <v>5.4</v>
+        <f>IFERROR(C11/'⚙ Configuración'!C12,0)</f>
+        <v>5.2</v>
       </c>
       <c r="D14" s="43" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E14" s="44"/>
     </row>
     <row r="15" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" s="49">
+        <f>IFERROR(C11/('⚙ Configuración'!C12*'⚙ Configuración'!C9),0)</f>
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E15" s="45"/>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="91" t="s">
         <v>128</v>
       </c>
-      <c r="C15" s="49">
-        <f>IFERROR('📋 Sprint Backlog'!G27/('⚙ Configuración'!C12*'⚙ Configuración'!C9),0)</f>
-        <v>0.9</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E15" s="45"/>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="75" t="s">
-        <v>130</v>
-      </c>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="68"/>
+      <c r="C16" s="72"/>
+      <c r="D16" s="72"/>
+      <c r="E16" s="73"/>
     </row>
     <row r="17" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C17" s="42">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E17" s="45"/>
     </row>
     <row r="18" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="41" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C18" s="42">
-        <f>'⚙ Configuración'!C9-C17</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D18" s="43" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E18" s="44"/>
     </row>
     <row r="19" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C19" s="48">
-        <f>IF(C18&lt;=0,"Sprint terminado",('📋 Sprint Backlog'!F27-'📋 Sprint Backlog'!G27)/C18)</f>
-        <v>8.1666666666666661</v>
+        <v>133</v>
+      </c>
+      <c r="C19" s="48" t="str">
+        <f>IF(C18&lt;=0,"Sprint terminado",('📋 Sprint Backlog'!F28-'📋 Sprint Backlog'!G28)/C18)</f>
+        <v>Sprint terminado</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E19" s="45"/>
     </row>
     <row r="20" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="41" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C20" s="48">
-        <f>IF(C17=0,0,'📋 Sprint Backlog'!G27/C17)</f>
-        <v>0</v>
+        <f>IF(C17=0,0,'📋 Sprint Backlog'!G28/C17)</f>
+        <v>7</v>
       </c>
       <c r="D20" s="43" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E20" s="44"/>
     </row>
     <row r="21" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C21" s="49">
         <f>IF(C17=0,1,C20/IFERROR(('⚙ Configuración'!C10/'⚙ Configuración'!C9),1))</f>
-        <v>1</v>
+        <v>0.55263157894736847</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E21" s="45"/>
     </row>
     <row r="22" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="76" t="s">
-        <v>141</v>
-      </c>
-      <c r="C22" s="67"/>
-      <c r="D22" s="67"/>
-      <c r="E22" s="68"/>
+      <c r="B22" s="92" t="s">
+        <v>139</v>
+      </c>
+      <c r="C22" s="72"/>
+      <c r="D22" s="72"/>
+      <c r="E22" s="73"/>
     </row>
     <row r="23" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="51" t="s">
-        <v>142</v>
-      </c>
-      <c r="C23" s="77" t="s">
-        <v>143</v>
-      </c>
-      <c r="D23" s="67"/>
-      <c r="E23" s="68"/>
+        <v>140</v>
+      </c>
+      <c r="C23" s="93" t="s">
+        <v>141</v>
+      </c>
+      <c r="D23" s="72"/>
+      <c r="E23" s="73"/>
     </row>
     <row r="24" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="52" t="s">
-        <v>144</v>
-      </c>
-      <c r="C24" s="66" t="s">
-        <v>145</v>
-      </c>
-      <c r="D24" s="67"/>
-      <c r="E24" s="68"/>
+        <v>142</v>
+      </c>
+      <c r="C24" s="88" t="s">
+        <v>143</v>
+      </c>
+      <c r="D24" s="72"/>
+      <c r="E24" s="73"/>
     </row>
     <row r="25" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="53" t="s">
-        <v>146</v>
-      </c>
-      <c r="C25" s="69" t="s">
-        <v>147</v>
-      </c>
-      <c r="D25" s="67"/>
-      <c r="E25" s="68"/>
+        <v>144</v>
+      </c>
+      <c r="C25" s="89" t="s">
+        <v>145</v>
+      </c>
+      <c r="D25" s="72"/>
+      <c r="E25" s="73"/>
     </row>
     <row r="26" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="C26" s="70" t="s">
-        <v>149</v>
-      </c>
-      <c r="D26" s="67"/>
-      <c r="E26" s="68"/>
+        <v>146</v>
+      </c>
+      <c r="C26" s="90" t="s">
+        <v>147</v>
+      </c>
+      <c r="D26" s="72"/>
+      <c r="E26" s="73"/>
     </row>
     <row r="27" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15724,171 +15789,165 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="3" customWidth="1"/>
-    <col min="3" max="3" width="67.28515625" customWidth="1"/>
+    <col min="3" max="3" width="75.28515625" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" customWidth="1"/>
     <col min="6" max="6" width="3" customWidth="1"/>
     <col min="7" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:5" ht="21" x14ac:dyDescent="0.25">
       <c r="C1" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="D1" s="72"/>
+      <c r="E1" s="73"/>
+    </row>
+    <row r="2" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C2" s="96" t="s">
+        <v>172</v>
+      </c>
+      <c r="D2" s="72"/>
+      <c r="E2" s="73"/>
+    </row>
+    <row r="3" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C3" s="97" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" s="72"/>
+      <c r="E3" s="73"/>
+    </row>
+    <row r="4" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C4" s="93" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="67"/>
-      <c r="E1" s="68"/>
-    </row>
-    <row r="2" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C2" s="72" t="s">
+      <c r="D4" s="72"/>
+      <c r="E4" s="73"/>
+    </row>
+    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C5" s="93" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" s="72"/>
+      <c r="E5" s="73"/>
+    </row>
+    <row r="6" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C6" s="93"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="73"/>
+    </row>
+    <row r="8" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C8" s="98" t="s">
         <v>151</v>
       </c>
-      <c r="D2" s="67"/>
-      <c r="E2" s="68"/>
-    </row>
-    <row r="3" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C3" s="90" t="s">
+      <c r="D8" s="72"/>
+      <c r="E8" s="73"/>
+    </row>
+    <row r="9" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C9" s="99" t="s">
+        <v>173</v>
+      </c>
+      <c r="D9" s="72"/>
+      <c r="E9" s="73"/>
+    </row>
+    <row r="10" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C10" s="99" t="s">
+        <v>175</v>
+      </c>
+      <c r="D10" s="72"/>
+      <c r="E10" s="73"/>
+    </row>
+    <row r="11" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C11" s="90"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="73"/>
+    </row>
+    <row r="13" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C13" s="100" t="s">
         <v>152</v>
       </c>
-      <c r="D3" s="67"/>
-      <c r="E3" s="68"/>
-    </row>
-    <row r="4" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C4" s="77" t="s">
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
+    </row>
+    <row r="14" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C14" s="94" t="s">
+        <v>177</v>
+      </c>
+      <c r="D14" s="72"/>
+      <c r="E14" s="73"/>
+    </row>
+    <row r="15" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C15" s="94" t="s">
+        <v>174</v>
+      </c>
+      <c r="D15" s="72"/>
+      <c r="E15" s="73"/>
+    </row>
+    <row r="16" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C16" s="88"/>
+      <c r="D16" s="72"/>
+      <c r="E16" s="73"/>
+    </row>
+    <row r="18" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C18" s="95" t="s">
         <v>153</v>
       </c>
-      <c r="D4" s="67"/>
-      <c r="E4" s="68"/>
-    </row>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C5" s="77" t="s">
-        <v>154</v>
-      </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="68"/>
-    </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C6" s="77" t="s">
-        <v>155</v>
-      </c>
-      <c r="D6" s="67"/>
-      <c r="E6" s="68"/>
-    </row>
-    <row r="8" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C8" s="91" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" s="67"/>
-      <c r="E8" s="68"/>
-    </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C9" s="70" t="s">
-        <v>157</v>
-      </c>
-      <c r="D9" s="67"/>
-      <c r="E9" s="68"/>
-    </row>
-    <row r="10" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C10" s="70" t="s">
-        <v>158</v>
-      </c>
-      <c r="D10" s="67"/>
-      <c r="E10" s="68"/>
-    </row>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C11" s="70" t="s">
-        <v>155</v>
-      </c>
-      <c r="D11" s="67"/>
-      <c r="E11" s="68"/>
-    </row>
-    <row r="13" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C13" s="92" t="s">
-        <v>159</v>
-      </c>
-      <c r="D13" s="67"/>
-      <c r="E13" s="68"/>
-    </row>
-    <row r="14" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C14" s="66" t="s">
-        <v>160</v>
-      </c>
-      <c r="D14" s="67"/>
-      <c r="E14" s="68"/>
-    </row>
-    <row r="15" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C15" s="66" t="s">
-        <v>161</v>
-      </c>
-      <c r="D15" s="67"/>
-      <c r="E15" s="68"/>
-    </row>
-    <row r="16" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C16" s="66" t="s">
-        <v>162</v>
-      </c>
-      <c r="D16" s="67"/>
-      <c r="E16" s="68"/>
-    </row>
-    <row r="18" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C18" s="89" t="s">
-        <v>163</v>
-      </c>
-      <c r="D18" s="67"/>
-      <c r="E18" s="68"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="73"/>
     </row>
     <row r="19" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C19" s="56" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="D19" s="57" t="s">
         <v>24</v>
       </c>
       <c r="E19" s="58" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="3:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="59" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D20" s="60" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="E20" s="61">
-        <v>46303</v>
+        <v>46324</v>
       </c>
     </row>
     <row r="21" spans="3:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="62" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="D21" s="63" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E21" s="64">
-        <v>46303</v>
+        <v>46317</v>
       </c>
     </row>
     <row r="22" spans="3:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="59" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="D22" s="60" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="E22" s="61">
-        <v>46303</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="23" spans="3:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="62" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="D23" s="63" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E23" s="65">
-        <v>46291</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="24" spans="3:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
docs(scrum): agregar columna de story points comprometidos por sprint en configuración
</commit_message>
<xml_diff>
--- a/scrum/burndown/PubTube_Burndown_B_S2.xlsx
+++ b/scrum/burndown/PubTube_Burndown_B_S2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccien\Documents\github\PubTube-Modulo2\scrum\burndown\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6AC42B-5358-4EDA-B56E-8FAD48D4BE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5166270-74FF-47F1-B5BB-C5C31C6C7463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5145" yWindow="2355" windowWidth="21600" windowHeight="11385" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="⚙ Configuración" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="181">
   <si>
     <t>🏃  Configuración del Sprint</t>
   </si>
@@ -639,6 +639,15 @@
   </si>
   <si>
     <t xml:space="preserve">  •  redistribuir de mejor manera los SPs de las historias de usuario a lo largo del tiempo</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>SP acumulado</t>
+  </si>
+  <si>
+    <t>Story Points comprometidos (sprint)</t>
   </si>
 </sst>
 </file>
@@ -1094,7 +1103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1294,18 +1303,48 @@
     <xf numFmtId="0" fontId="36" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1319,28 +1358,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5648,7 +5666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:D1000"/>
+  <dimension ref="B1:D1001"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -5660,25 +5678,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="72"/>
-      <c r="D1" s="73"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="76"/>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="76"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="81" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="72"/>
-      <c r="D3" s="73"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="76"/>
     </row>
     <row r="4" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
@@ -5736,104 +5754,112 @@
     </row>
     <row r="10" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C10" s="72">
+        <v>29</v>
+      </c>
+      <c r="D10" s="73"/>
+    </row>
+    <row r="11" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C11" s="2">
         <f>'📋 Sprint Backlog'!F28</f>
         <v>76</v>
       </c>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="2">
-        <v>16</v>
-      </c>
       <c r="D11" s="3"/>
     </row>
     <row r="12" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="2">
+        <v>16</v>
+      </c>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C13" s="2">
         <v>5</v>
       </c>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="86" t="s">
+      <c r="D13" s="3"/>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="72"/>
-      <c r="D13" s="73"/>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="75" t="s">
+      <c r="C14" s="75"/>
+      <c r="D14" s="76"/>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="72"/>
-      <c r="D14" s="73"/>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="75" t="s">
+      <c r="C15" s="75"/>
+      <c r="D15" s="76"/>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="72"/>
-      <c r="D15" s="73"/>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="75" t="s">
+      <c r="C16" s="75"/>
+      <c r="D16" s="76"/>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="72"/>
-      <c r="D16" s="73"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="75" t="s">
+      <c r="C17" s="75"/>
+      <c r="D17" s="76"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="72"/>
-      <c r="D17" s="73"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="75" t="s">
+      <c r="C18" s="75"/>
+      <c r="D18" s="76"/>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="72"/>
-      <c r="D18" s="73"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="76" t="s">
+      <c r="C19" s="75"/>
+      <c r="D19" s="76"/>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="72"/>
-      <c r="D19" s="73"/>
-    </row>
-    <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="77" t="s">
+      <c r="C20" s="75"/>
+      <c r="D20" s="76"/>
+    </row>
+    <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="87" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="78"/>
-      <c r="D20" s="79"/>
-    </row>
-    <row r="21" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="80"/>
-      <c r="C21" s="81"/>
-      <c r="D21" s="82"/>
+      <c r="C21" s="88"/>
+      <c r="D21" s="89"/>
     </row>
     <row r="22" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="80"/>
-      <c r="C22" s="81"/>
-      <c r="D22" s="82"/>
+      <c r="B22" s="90"/>
+      <c r="C22" s="91"/>
+      <c r="D22" s="92"/>
     </row>
     <row r="23" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="83"/>
-      <c r="C23" s="84"/>
-      <c r="D23" s="85"/>
-    </row>
-    <row r="24" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B23" s="90"/>
+      <c r="C23" s="91"/>
+      <c r="D23" s="92"/>
+    </row>
+    <row r="24" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="93"/>
+      <c r="C24" s="94"/>
+      <c r="D24" s="95"/>
+    </row>
     <row r="25" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6810,19 +6836,20 @@
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B20:D23"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D24"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -6847,28 +6874,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="73"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="76"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="76"/>
     </row>
     <row r="3" spans="2:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
@@ -6939,6 +6966,7 @@
         <v>3</v>
       </c>
       <c r="G5" s="15">
+        <f t="shared" ref="G5:G22" si="0">IF(H5="Done",F5,"")</f>
         <v>3</v>
       </c>
       <c r="H5" s="16" t="s">
@@ -6965,6 +6993,7 @@
         <v>3</v>
       </c>
       <c r="G6" s="15">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H6" s="16" t="s">
@@ -6991,6 +7020,7 @@
         <v>2</v>
       </c>
       <c r="G7" s="15">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="H7" s="16" t="s">
@@ -7017,6 +7047,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="15">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H8" s="16" t="s">
@@ -7043,6 +7074,7 @@
         <v>3</v>
       </c>
       <c r="G9" s="15">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H9" s="16" t="s">
@@ -7069,6 +7101,7 @@
         <v>3</v>
       </c>
       <c r="G10" s="15">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H10" s="16" t="s">
@@ -7095,6 +7128,7 @@
         <v>2</v>
       </c>
       <c r="G11" s="15">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="H11" s="16" t="s">
@@ -7118,7 +7152,10 @@
       <c r="F12" s="14">
         <v>5</v>
       </c>
-      <c r="G12" s="15"/>
+      <c r="G12" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H12" s="16" t="s">
         <v>52</v>
       </c>
@@ -7140,7 +7177,10 @@
       <c r="F13" s="14">
         <v>3</v>
       </c>
-      <c r="G13" s="15"/>
+      <c r="G13" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H13" s="16" t="s">
         <v>52</v>
       </c>
@@ -7165,6 +7205,7 @@
         <v>3</v>
       </c>
       <c r="G14" s="15">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H14" s="16" t="s">
@@ -7190,7 +7231,8 @@
       <c r="F15" s="14">
         <v>3</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="15">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H15" s="16" t="s">
@@ -7214,7 +7256,10 @@
       <c r="F16" s="14">
         <v>5</v>
       </c>
-      <c r="G16" s="15"/>
+      <c r="G16" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H16" s="16" t="s">
         <v>52</v>
       </c>
@@ -7237,7 +7282,10 @@
       <c r="F17" s="14">
         <v>3</v>
       </c>
-      <c r="G17" s="15"/>
+      <c r="G17" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H17" s="16" t="s">
         <v>52</v>
       </c>
@@ -7259,7 +7307,10 @@
       <c r="F18" s="14">
         <v>3</v>
       </c>
-      <c r="G18" s="15"/>
+      <c r="G18" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H18" s="16" t="s">
         <v>52</v>
       </c>
@@ -7281,7 +7332,10 @@
       <c r="F19" s="14">
         <v>2</v>
       </c>
-      <c r="G19" s="15"/>
+      <c r="G19" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H19" s="16" t="s">
         <v>52</v>
       </c>
@@ -7303,7 +7357,10 @@
       <c r="F20" s="14">
         <v>5</v>
       </c>
-      <c r="G20" s="15"/>
+      <c r="G20" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H20" s="16" t="s">
         <v>52</v>
       </c>
@@ -7325,7 +7382,10 @@
       <c r="F21" s="14">
         <v>3</v>
       </c>
-      <c r="G21" s="15"/>
+      <c r="G21" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="H21" s="16" t="s">
         <v>52</v>
       </c>
@@ -7350,6 +7410,7 @@
         <v>3</v>
       </c>
       <c r="G22" s="15">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H22" s="16" t="s">
@@ -7376,6 +7437,7 @@
         <v>2</v>
       </c>
       <c r="G23" s="15">
+        <f t="shared" ref="G23:G27" si="1">IF(H23="Done",F23,"")</f>
         <v>2</v>
       </c>
       <c r="H23" s="16" t="s">
@@ -7402,6 +7464,7 @@
         <v>2</v>
       </c>
       <c r="G24" s="15">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="H24" s="16" t="s">
@@ -7428,6 +7491,7 @@
         <v>3</v>
       </c>
       <c r="G25" s="15">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H25" s="16" t="s">
@@ -7451,7 +7515,10 @@
       <c r="F26" s="14">
         <v>2</v>
       </c>
-      <c r="G26" s="15"/>
+      <c r="G26" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="H26" s="16" t="s">
         <v>52</v>
       </c>
@@ -7473,7 +7540,10 @@
       <c r="F27" s="14">
         <v>3</v>
       </c>
-      <c r="G27" s="15"/>
+      <c r="G27" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="H27" s="16" t="s">
         <v>52</v>
       </c>
@@ -7482,18 +7552,18 @@
       </c>
     </row>
     <row r="28" spans="2:9" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B28" s="87" t="s">
+      <c r="B28" s="96" t="s">
         <v>87</v>
       </c>
-      <c r="C28" s="72"/>
-      <c r="D28" s="72"/>
-      <c r="E28" s="73"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="75"/>
+      <c r="E28" s="76"/>
       <c r="F28" s="19">
-        <f t="shared" ref="F28:G28" si="0">SUM(F4:F27)</f>
+        <f t="shared" ref="F28:G28" si="2">SUM(F4:F27)</f>
         <v>76</v>
       </c>
       <c r="G28" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>42</v>
       </c>
       <c r="H28" s="21">
@@ -10499,26 +10569,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="79" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="73"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="76"/>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="80" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="76"/>
     </row>
     <row r="3" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="24" t="s">
@@ -10566,7 +10636,7 @@
         <v>46265</v>
       </c>
       <c r="E4" s="29">
-        <f>IF($B4&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B4) / 24)</f>
+        <f>IF($B4&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B4) / 24)</f>
         <v>76</v>
       </c>
       <c r="F4" s="15"/>
@@ -10575,12 +10645,12 @@
         <v>0</v>
       </c>
       <c r="H4" s="36">
-        <f>'⚙ Configuración'!$C$10-G4</f>
+        <f>'⚙ Configuración'!$C$11-G4</f>
         <v>76</v>
       </c>
       <c r="I4" s="37"/>
       <c r="J4" s="38">
-        <f>IF($B4&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B4 - 1) / 24)</f>
+        <f>IF($B4&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B4 - 1) / 24)</f>
         <v>0</v>
       </c>
       <c r="K4" s="39">
@@ -10601,7 +10671,7 @@
         <v>46268</v>
       </c>
       <c r="E5" s="29">
-        <f>IF($B5&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B5) / 24)</f>
+        <f>IF($B5&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B5) / 24)</f>
         <v>72.833333333333329</v>
       </c>
       <c r="F5" s="15"/>
@@ -10610,12 +10680,12 @@
         <v>0</v>
       </c>
       <c r="H5" s="36">
-        <f>'⚙ Configuración'!$C$10-G5</f>
+        <f>'⚙ Configuración'!$C$11-G5</f>
         <v>76</v>
       </c>
       <c r="I5" s="37"/>
       <c r="J5" s="38">
-        <f>IF($B5&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B5 - 1) / 24)</f>
+        <f>IF($B5&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B5 - 1) / 24)</f>
         <v>3.1666666666666665</v>
       </c>
       <c r="K5" s="67"/>
@@ -10632,7 +10702,7 @@
         <v>46272</v>
       </c>
       <c r="E6" s="29">
-        <f>IF($B6&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B6) / 24)</f>
+        <f>IF($B6&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B6) / 24)</f>
         <v>69.666666666666671</v>
       </c>
       <c r="F6" s="15">
@@ -10644,12 +10714,12 @@
         <v>5</v>
       </c>
       <c r="H6" s="36">
-        <f>'⚙ Configuración'!$C$10-G6</f>
+        <f>'⚙ Configuración'!$C$11-G6</f>
         <v>71</v>
       </c>
       <c r="I6" s="37"/>
       <c r="J6" s="38">
-        <f>IF($B6&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B6 - 1) / 24)</f>
+        <f>IF($B6&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B6 - 1) / 24)</f>
         <v>6.333333333333333</v>
       </c>
       <c r="K6" s="67"/>
@@ -10666,7 +10736,7 @@
         <v>46275</v>
       </c>
       <c r="E7" s="29">
-        <f>IF($B7&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B7) / 24)</f>
+        <f>IF($B7&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B7) / 24)</f>
         <v>66.5</v>
       </c>
       <c r="F7" s="15">
@@ -10678,12 +10748,12 @@
         <v>16</v>
       </c>
       <c r="H7" s="36">
-        <f>'⚙ Configuración'!$C$10-G7</f>
+        <f>'⚙ Configuración'!$C$11-G7</f>
         <v>60</v>
       </c>
       <c r="I7" s="37"/>
       <c r="J7" s="38">
-        <f>IF($B7&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B7 - 1) / 24)</f>
+        <f>IF($B7&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B7 - 1) / 24)</f>
         <v>9.5</v>
       </c>
       <c r="K7" s="67"/>
@@ -10703,7 +10773,7 @@
         <v>46279</v>
       </c>
       <c r="E8" s="29">
-        <f>IF($B8&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B8) / 24)</f>
+        <f>IF($B8&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B8) / 24)</f>
         <v>63.333333333333336</v>
       </c>
       <c r="F8" s="15"/>
@@ -10712,12 +10782,12 @@
         <v>16</v>
       </c>
       <c r="H8" s="36">
-        <f>'⚙ Configuración'!$C$10-G8</f>
+        <f>'⚙ Configuración'!$C$11-G8</f>
         <v>60</v>
       </c>
       <c r="I8" s="37"/>
       <c r="J8" s="38">
-        <f>IF($B8&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B8 - 1) / 24)</f>
+        <f>IF($B8&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B8 - 1) / 24)</f>
         <v>12.666666666666666</v>
       </c>
       <c r="K8" s="67"/>
@@ -10737,7 +10807,7 @@
         <v>46282</v>
       </c>
       <c r="E9" s="29">
-        <f>IF($B9&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B9) / 24)</f>
+        <f>IF($B9&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B9) / 24)</f>
         <v>60.166666666666664</v>
       </c>
       <c r="F9" s="15"/>
@@ -10746,15 +10816,15 @@
         <v>16</v>
       </c>
       <c r="H9" s="36">
-        <f>'⚙ Configuración'!$C$10-G9</f>
+        <f>'⚙ Configuración'!$C$11-G9</f>
         <v>60</v>
       </c>
       <c r="I9" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J9" s="38">
-        <f>IF($B9&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B9 - 1) / 24)</f>
+        <f>IF($B9&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B9 - 1) / 24)</f>
         <v>15.833333333333334</v>
       </c>
       <c r="K9" s="23">
@@ -10778,7 +10848,7 @@
         <v>46286</v>
       </c>
       <c r="E10" s="29">
-        <f>IF($B10&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B10) / 24)</f>
+        <f>IF($B10&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B10) / 24)</f>
         <v>57</v>
       </c>
       <c r="F10" s="15"/>
@@ -10787,12 +10857,12 @@
         <v>16</v>
       </c>
       <c r="H10" s="36">
-        <f>'⚙ Configuración'!$C$10-G10</f>
+        <f>'⚙ Configuración'!$C$11-G10</f>
         <v>60</v>
       </c>
       <c r="I10" s="37"/>
       <c r="J10" s="38">
-        <f>IF($B10&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B10 - 1) / 24)</f>
+        <f>IF($B10&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B10 - 1) / 24)</f>
         <v>19</v>
       </c>
       <c r="K10" s="39"/>
@@ -10810,7 +10880,7 @@
         <v>46289</v>
       </c>
       <c r="E11" s="29">
-        <f>IF($B11&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B11) / 24)</f>
+        <f>IF($B11&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B11) / 24)</f>
         <v>53.833333333333336</v>
       </c>
       <c r="F11" s="15"/>
@@ -10819,12 +10889,12 @@
         <v>16</v>
       </c>
       <c r="H11" s="36">
-        <f>'⚙ Configuración'!$C$10-G11</f>
+        <f>'⚙ Configuración'!$C$11-G11</f>
         <v>60</v>
       </c>
       <c r="I11" s="37"/>
       <c r="J11" s="38">
-        <f>IF($B11&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B11 - 1) / 24)</f>
+        <f>IF($B11&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B11 - 1) / 24)</f>
         <v>22.166666666666668</v>
       </c>
       <c r="K11" s="39"/>
@@ -10842,7 +10912,7 @@
         <v>46293</v>
       </c>
       <c r="E12" s="29">
-        <f>IF($B12&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B12) / 24)</f>
+        <f>IF($B12&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B12) / 24)</f>
         <v>50.666666666666664</v>
       </c>
       <c r="F12" s="15"/>
@@ -10851,12 +10921,12 @@
         <v>16</v>
       </c>
       <c r="H12" s="36">
-        <f>'⚙ Configuración'!$C$10-G12</f>
+        <f>'⚙ Configuración'!$C$11-G12</f>
         <v>60</v>
       </c>
       <c r="I12" s="37"/>
       <c r="J12" s="38">
-        <f>IF($B12&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B12 - 1) / 24)</f>
+        <f>IF($B12&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B12 - 1) / 24)</f>
         <v>25.333333333333332</v>
       </c>
       <c r="K12" s="39"/>
@@ -10874,7 +10944,7 @@
         <v>46296</v>
       </c>
       <c r="E13" s="29">
-        <f>IF($B13&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B13) / 24)</f>
+        <f>IF($B13&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B13) / 24)</f>
         <v>47.5</v>
       </c>
       <c r="F13" s="15"/>
@@ -10883,12 +10953,12 @@
         <v>16</v>
       </c>
       <c r="H13" s="36">
-        <f>'⚙ Configuración'!$C$10-G13</f>
+        <f>'⚙ Configuración'!$C$11-G13</f>
         <v>60</v>
       </c>
       <c r="I13" s="37"/>
       <c r="J13" s="38">
-        <f>IF($B13&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B13 - 1) / 24)</f>
+        <f>IF($B13&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B13 - 1) / 24)</f>
         <v>28.5</v>
       </c>
       <c r="K13" s="39"/>
@@ -10906,7 +10976,7 @@
         <v>46300</v>
       </c>
       <c r="E14" s="29">
-        <f>IF($B14&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B14) / 24)</f>
+        <f>IF($B14&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B14) / 24)</f>
         <v>44.333333333333336</v>
       </c>
       <c r="F14" s="15"/>
@@ -10915,12 +10985,12 @@
         <v>16</v>
       </c>
       <c r="H14" s="36">
-        <f>'⚙ Configuración'!$C$10-G14</f>
+        <f>'⚙ Configuración'!$C$11-G14</f>
         <v>60</v>
       </c>
       <c r="I14" s="37"/>
       <c r="J14" s="38">
-        <f>IF($B14&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B14 - 1) / 24)</f>
+        <f>IF($B14&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B14 - 1) / 24)</f>
         <v>31.666666666666668</v>
       </c>
       <c r="K14" s="39"/>
@@ -10938,7 +11008,7 @@
         <v>46303</v>
       </c>
       <c r="E15" s="29">
-        <f>IF($B15&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B15) / 24)</f>
+        <f>IF($B15&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B15) / 24)</f>
         <v>41.166666666666664</v>
       </c>
       <c r="F15" s="15"/>
@@ -10947,15 +11017,15 @@
         <v>16</v>
       </c>
       <c r="H15" s="36">
-        <f>'⚙ Configuración'!$C$10-G15</f>
+        <f>'⚙ Configuración'!$C$11-G15</f>
         <v>60</v>
       </c>
       <c r="I15" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J15" s="38">
-        <f>IF($B15&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B15 - 1) / 24)</f>
+        <f>IF($B15&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B15 - 1) / 24)</f>
         <v>34.833333333333336</v>
       </c>
       <c r="K15" s="39">
@@ -10977,7 +11047,7 @@
         <v>46307</v>
       </c>
       <c r="E16" s="29">
-        <f>IF($B16&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B16) / 24)</f>
+        <f>IF($B16&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B16) / 24)</f>
         <v>38</v>
       </c>
       <c r="F16" s="15"/>
@@ -10986,12 +11056,12 @@
         <v>16</v>
       </c>
       <c r="H16" s="36">
-        <f>'⚙ Configuración'!$C$10-G16</f>
+        <f>'⚙ Configuración'!$C$11-G16</f>
         <v>60</v>
       </c>
       <c r="I16" s="37"/>
       <c r="J16" s="38">
-        <f>IF($B16&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B16 - 1) / 24)</f>
+        <f>IF($B16&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B16 - 1) / 24)</f>
         <v>38</v>
       </c>
       <c r="K16" s="39"/>
@@ -11008,7 +11078,7 @@
         <v>46310</v>
       </c>
       <c r="E17" s="29">
-        <f>IF($B17&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B17) / 24)</f>
+        <f>IF($B17&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B17) / 24)</f>
         <v>34.833333333333336</v>
       </c>
       <c r="F17" s="15"/>
@@ -11017,12 +11087,12 @@
         <v>16</v>
       </c>
       <c r="H17" s="36">
-        <f>'⚙ Configuración'!$C$10-G17</f>
+        <f>'⚙ Configuración'!$C$11-G17</f>
         <v>60</v>
       </c>
       <c r="I17" s="37"/>
       <c r="J17" s="38">
-        <f>IF($B17&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B17 - 1) / 24)</f>
+        <f>IF($B17&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B17 - 1) / 24)</f>
         <v>41.166666666666664</v>
       </c>
       <c r="K17" s="39"/>
@@ -11039,7 +11109,7 @@
         <v>46314</v>
       </c>
       <c r="E18" s="29">
-        <f>IF($B18&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B18) / 24)</f>
+        <f>IF($B18&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B18) / 24)</f>
         <v>31.666666666666668</v>
       </c>
       <c r="F18" s="15"/>
@@ -11048,12 +11118,12 @@
         <v>16</v>
       </c>
       <c r="H18" s="36">
-        <f>'⚙ Configuración'!$C$10-G18</f>
+        <f>'⚙ Configuración'!$C$11-G18</f>
         <v>60</v>
       </c>
       <c r="I18" s="37"/>
       <c r="J18" s="38">
-        <f>IF($B18&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B18 - 1) / 24)</f>
+        <f>IF($B18&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B18 - 1) / 24)</f>
         <v>44.333333333333336</v>
       </c>
       <c r="K18" s="39"/>
@@ -11070,7 +11140,7 @@
         <v>46317</v>
       </c>
       <c r="E19" s="29">
-        <f>IF($B19&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B19) / 24)</f>
+        <f>IF($B19&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B19) / 24)</f>
         <v>28.5</v>
       </c>
       <c r="F19" s="15"/>
@@ -11079,12 +11149,12 @@
         <v>16</v>
       </c>
       <c r="H19" s="36">
-        <f>'⚙ Configuración'!$C$10-G19</f>
+        <f>'⚙ Configuración'!$C$11-G19</f>
         <v>60</v>
       </c>
       <c r="I19" s="37"/>
       <c r="J19" s="38">
-        <f>IF($B19&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B19 - 1) / 24)</f>
+        <f>IF($B19&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B19 - 1) / 24)</f>
         <v>47.5</v>
       </c>
       <c r="K19" s="39"/>
@@ -11101,7 +11171,7 @@
         <v>46321</v>
       </c>
       <c r="E20" s="29">
-        <f>IF($B20&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B20) / 24)</f>
+        <f>IF($B20&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B20) / 24)</f>
         <v>25.333333333333332</v>
       </c>
       <c r="F20" s="15"/>
@@ -11110,12 +11180,12 @@
         <v>16</v>
       </c>
       <c r="H20" s="36">
-        <f>'⚙ Configuración'!$C$10-G20</f>
+        <f>'⚙ Configuración'!$C$11-G20</f>
         <v>60</v>
       </c>
       <c r="I20" s="37"/>
       <c r="J20" s="38">
-        <f>IF($B20&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B20 - 1) / 24)</f>
+        <f>IF($B20&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B20 - 1) / 24)</f>
         <v>50.666666666666664</v>
       </c>
       <c r="K20" s="39"/>
@@ -11132,7 +11202,7 @@
         <v>46324</v>
       </c>
       <c r="E21" s="29">
-        <f>IF($B21&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B21) / 24)</f>
+        <f>IF($B21&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B21) / 24)</f>
         <v>22.166666666666668</v>
       </c>
       <c r="F21" s="15"/>
@@ -11141,15 +11211,15 @@
         <v>16</v>
       </c>
       <c r="H21" s="36">
-        <f>'⚙ Configuración'!$C$10-G21</f>
+        <f>'⚙ Configuración'!$C$11-G21</f>
         <v>60</v>
       </c>
       <c r="I21" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J21" s="38">
-        <f>IF($B21&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B21 - 1) / 24)</f>
+        <f>IF($B21&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B21 - 1) / 24)</f>
         <v>53.833333333333336</v>
       </c>
       <c r="K21" s="39">
@@ -11170,7 +11240,7 @@
         <v>46328</v>
       </c>
       <c r="E22" s="29">
-        <f>IF($B22&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B22) / 24)</f>
+        <f>IF($B22&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B22) / 24)</f>
         <v>19</v>
       </c>
       <c r="F22" s="15"/>
@@ -11179,12 +11249,12 @@
         <v>16</v>
       </c>
       <c r="H22" s="36">
-        <f>'⚙ Configuración'!$C$10-G22</f>
+        <f>'⚙ Configuración'!$C$11-G22</f>
         <v>60</v>
       </c>
       <c r="I22" s="37"/>
       <c r="J22" s="38">
-        <f>IF($B22&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B22 - 1) / 24)</f>
+        <f>IF($B22&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B22 - 1) / 24)</f>
         <v>57</v>
       </c>
       <c r="K22" s="39"/>
@@ -11201,7 +11271,7 @@
         <v>46331</v>
       </c>
       <c r="E23" s="29">
-        <f>IF($B23&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B23) / 24)</f>
+        <f>IF($B23&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B23) / 24)</f>
         <v>15.833333333333334</v>
       </c>
       <c r="F23" s="15"/>
@@ -11210,12 +11280,12 @@
         <v>16</v>
       </c>
       <c r="H23" s="36">
-        <f>'⚙ Configuración'!$C$10-G23</f>
+        <f>'⚙ Configuración'!$C$11-G23</f>
         <v>60</v>
       </c>
       <c r="I23" s="37"/>
       <c r="J23" s="38">
-        <f>IF($B23&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B23 - 1) / 24)</f>
+        <f>IF($B23&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B23 - 1) / 24)</f>
         <v>60.166666666666664</v>
       </c>
       <c r="K23" s="39"/>
@@ -11232,7 +11302,7 @@
         <v>46335</v>
       </c>
       <c r="E24" s="29">
-        <f>IF($B24&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B24) / 24)</f>
+        <f>IF($B24&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B24) / 24)</f>
         <v>12.666666666666666</v>
       </c>
       <c r="F24" s="15"/>
@@ -11241,12 +11311,12 @@
         <v>16</v>
       </c>
       <c r="H24" s="36">
-        <f>'⚙ Configuración'!$C$10-G24</f>
+        <f>'⚙ Configuración'!$C$11-G24</f>
         <v>60</v>
       </c>
       <c r="I24" s="37"/>
       <c r="J24" s="38">
-        <f>IF($B24&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B24 - 1) / 24)</f>
+        <f>IF($B24&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B24 - 1) / 24)</f>
         <v>63.333333333333336</v>
       </c>
       <c r="K24" s="39"/>
@@ -11263,7 +11333,7 @@
         <v>46338</v>
       </c>
       <c r="E25" s="29">
-        <f>IF($B25&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B25) / 24)</f>
+        <f>IF($B25&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B25) / 24)</f>
         <v>9.5</v>
       </c>
       <c r="F25" s="15"/>
@@ -11272,12 +11342,12 @@
         <v>16</v>
       </c>
       <c r="H25" s="36">
-        <f>'⚙ Configuración'!$C$10-G25</f>
+        <f>'⚙ Configuración'!$C$11-G25</f>
         <v>60</v>
       </c>
       <c r="I25" s="37"/>
       <c r="J25" s="38">
-        <f>IF($B25&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B25 - 1) / 24)</f>
+        <f>IF($B25&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B25 - 1) / 24)</f>
         <v>66.5</v>
       </c>
       <c r="K25" s="39"/>
@@ -11294,7 +11364,7 @@
         <v>46335</v>
       </c>
       <c r="E26" s="29">
-        <f>IF($B26&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B26) / 24)</f>
+        <f>IF($B26&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B26) / 24)</f>
         <v>6.333333333333333</v>
       </c>
       <c r="F26" s="15"/>
@@ -11303,12 +11373,12 @@
         <v>16</v>
       </c>
       <c r="H26" s="36">
-        <f>'⚙ Configuración'!$C$10-G26</f>
+        <f>'⚙ Configuración'!$C$11-G26</f>
         <v>60</v>
       </c>
       <c r="I26" s="37"/>
       <c r="J26" s="38">
-        <f>IF($B26&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B26 - 1) / 24)</f>
+        <f>IF($B26&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B26 - 1) / 24)</f>
         <v>69.666666666666671</v>
       </c>
       <c r="K26" s="39"/>
@@ -11325,7 +11395,7 @@
         <v>46342</v>
       </c>
       <c r="E27" s="29">
-        <f>IF($B27&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B27) / 24)</f>
+        <f>IF($B27&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B27) / 24)</f>
         <v>3.1666666666666665</v>
       </c>
       <c r="F27" s="15"/>
@@ -11334,12 +11404,12 @@
         <v>16</v>
       </c>
       <c r="H27" s="36">
-        <f>'⚙ Configuración'!$C$10-G27</f>
+        <f>'⚙ Configuración'!$C$11-G27</f>
         <v>60</v>
       </c>
       <c r="I27" s="37"/>
       <c r="J27" s="38">
-        <f>IF($B27&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B27 - 1) / 24)</f>
+        <f>IF($B27&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B27 - 1) / 24)</f>
         <v>72.833333333333329</v>
       </c>
       <c r="K27" s="39"/>
@@ -11356,7 +11426,7 @@
         <v>46345</v>
       </c>
       <c r="E28" s="29">
-        <f>IF($B28&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B28) / 24)</f>
+        <f>IF($B28&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B28) / 24)</f>
         <v>0</v>
       </c>
       <c r="F28" s="15"/>
@@ -11365,19 +11435,19 @@
         <v>16</v>
       </c>
       <c r="H28" s="36">
-        <f>'⚙ Configuración'!$C$10-G28</f>
+        <f>'⚙ Configuración'!$C$11-G28</f>
         <v>60</v>
       </c>
       <c r="I28" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J28" s="38">
-        <f>IF($B28&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B28 - 1) / 24)</f>
+        <f>IF($B28&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B28 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K28" s="39">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="L28" s="39">
@@ -11395,7 +11465,7 @@
         <v>46349</v>
       </c>
       <c r="E29" s="29">
-        <f>IF($B29&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B29) / 24)</f>
+        <f>IF($B29&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B29) / 24)</f>
         <v>0</v>
       </c>
       <c r="F29" s="15"/>
@@ -11404,12 +11474,12 @@
         <v>16</v>
       </c>
       <c r="H29" s="36">
-        <f>'⚙ Configuración'!$C$10-G29</f>
+        <f>'⚙ Configuración'!$C$11-G29</f>
         <v>60</v>
       </c>
       <c r="I29" s="37"/>
       <c r="J29" s="38">
-        <f>IF($B29&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B29 - 1) / 24)</f>
+        <f>IF($B29&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B29 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K29" s="39"/>
@@ -11426,7 +11496,7 @@
         <v>46352</v>
       </c>
       <c r="E30" s="29">
-        <f>IF($B30&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B30) / 24)</f>
+        <f>IF($B30&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B30) / 24)</f>
         <v>0</v>
       </c>
       <c r="F30" s="15"/>
@@ -11435,12 +11505,12 @@
         <v>16</v>
       </c>
       <c r="H30" s="36">
-        <f>'⚙ Configuración'!$C$10-G30</f>
+        <f>'⚙ Configuración'!$C$11-G30</f>
         <v>60</v>
       </c>
       <c r="I30" s="37"/>
       <c r="J30" s="38">
-        <f>IF($B30&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B30 - 1) / 24)</f>
+        <f>IF($B30&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B30 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K30" s="39"/>
@@ -11457,7 +11527,7 @@
         <v>46356</v>
       </c>
       <c r="E31" s="29">
-        <f>IF($B31&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B31) / 24)</f>
+        <f>IF($B31&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B31) / 24)</f>
         <v>0</v>
       </c>
       <c r="F31" s="15"/>
@@ -11466,15 +11536,15 @@
         <v>16</v>
       </c>
       <c r="H31" s="36">
-        <f>'⚙ Configuración'!$C$10-G31</f>
+        <f>'⚙ Configuración'!$C$11-G31</f>
         <v>60</v>
       </c>
       <c r="I31" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J31" s="38">
-        <f>IF($B31&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B31 - 1) / 24)</f>
+        <f>IF($B31&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B31 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K31" s="39"/>
@@ -12484,26 +12554,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="79" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="73"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="76"/>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="80" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="76"/>
     </row>
     <row r="3" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="24" t="s">
@@ -12551,7 +12621,7 @@
         <v>46265</v>
       </c>
       <c r="E4" s="29">
-        <f>IF($B4&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B4) / 24)</f>
+        <f>IF($B4&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B4) / 24)</f>
         <v>76</v>
       </c>
       <c r="F4" s="15"/>
@@ -12560,12 +12630,12 @@
         <v>0</v>
       </c>
       <c r="H4" s="36">
-        <f>'⚙ Configuración'!$C$10-G4</f>
+        <f>'⚙ Configuración'!$C$11-G4</f>
         <v>76</v>
       </c>
       <c r="I4" s="37"/>
       <c r="J4" s="38">
-        <f>IF($B4&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B4 - 1) / 24)</f>
+        <f>IF($B4&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B4 - 1) / 24)</f>
         <v>0</v>
       </c>
       <c r="K4" s="39">
@@ -12586,7 +12656,7 @@
         <v>46268</v>
       </c>
       <c r="E5" s="29">
-        <f>IF($B5&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B5) / 24)</f>
+        <f>IF($B5&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B5) / 24)</f>
         <v>72.833333333333329</v>
       </c>
       <c r="F5" s="15"/>
@@ -12595,12 +12665,12 @@
         <v>0</v>
       </c>
       <c r="H5" s="36">
-        <f>'⚙ Configuración'!$C$10-G5</f>
+        <f>'⚙ Configuración'!$C$11-G5</f>
         <v>76</v>
       </c>
       <c r="I5" s="37"/>
       <c r="J5" s="38">
-        <f>IF($B5&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B5 - 1) / 24)</f>
+        <f>IF($B5&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B5 - 1) / 24)</f>
         <v>3.1666666666666665</v>
       </c>
       <c r="K5" s="39"/>
@@ -12617,7 +12687,7 @@
         <v>46272</v>
       </c>
       <c r="E6" s="29">
-        <f>IF($B6&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B6) / 24)</f>
+        <f>IF($B6&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B6) / 24)</f>
         <v>69.666666666666671</v>
       </c>
       <c r="F6" s="15">
@@ -12629,12 +12699,12 @@
         <v>5</v>
       </c>
       <c r="H6" s="36">
-        <f>'⚙ Configuración'!$C$10-G6</f>
+        <f>'⚙ Configuración'!$C$11-G6</f>
         <v>71</v>
       </c>
       <c r="I6" s="37"/>
       <c r="J6" s="38">
-        <f>IF($B6&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B6 - 1) / 24)</f>
+        <f>IF($B6&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B6 - 1) / 24)</f>
         <v>6.333333333333333</v>
       </c>
       <c r="K6" s="39"/>
@@ -12651,7 +12721,7 @@
         <v>46275</v>
       </c>
       <c r="E7" s="29">
-        <f>IF($B7&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B7) / 24)</f>
+        <f>IF($B7&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B7) / 24)</f>
         <v>66.5</v>
       </c>
       <c r="F7" s="15">
@@ -12663,12 +12733,12 @@
         <v>16</v>
       </c>
       <c r="H7" s="36">
-        <f>'⚙ Configuración'!$C$10-G7</f>
+        <f>'⚙ Configuración'!$C$11-G7</f>
         <v>60</v>
       </c>
       <c r="I7" s="37"/>
       <c r="J7" s="38">
-        <f>IF($B7&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B7 - 1) / 24)</f>
+        <f>IF($B7&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B7 - 1) / 24)</f>
         <v>9.5</v>
       </c>
       <c r="K7" s="39"/>
@@ -12686,7 +12756,7 @@
         <v>46279</v>
       </c>
       <c r="E8" s="29">
-        <f>IF($B8&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B8) / 24)</f>
+        <f>IF($B8&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B8) / 24)</f>
         <v>63.333333333333336</v>
       </c>
       <c r="F8" s="15"/>
@@ -12695,12 +12765,12 @@
         <v>16</v>
       </c>
       <c r="H8" s="36">
-        <f>'⚙ Configuración'!$C$10-G8</f>
+        <f>'⚙ Configuración'!$C$11-G8</f>
         <v>60</v>
       </c>
       <c r="I8" s="37"/>
       <c r="J8" s="38">
-        <f>IF($B8&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B8 - 1) / 24)</f>
+        <f>IF($B8&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B8 - 1) / 24)</f>
         <v>12.666666666666666</v>
       </c>
       <c r="K8" s="39"/>
@@ -12720,7 +12790,7 @@
         <v>46282</v>
       </c>
       <c r="E9" s="29">
-        <f>IF($B9&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B9) / 24)</f>
+        <f>IF($B9&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B9) / 24)</f>
         <v>60.166666666666664</v>
       </c>
       <c r="F9" s="15"/>
@@ -12729,15 +12799,15 @@
         <v>16</v>
       </c>
       <c r="H9" s="36">
-        <f>'⚙ Configuración'!$C$10-G9</f>
+        <f>'⚙ Configuración'!$C$11-G9</f>
         <v>60</v>
       </c>
       <c r="I9" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J9" s="38">
-        <f>IF($B9&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B9 - 1) / 24)</f>
+        <f>IF($B9&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B9 - 1) / 24)</f>
         <v>15.833333333333334</v>
       </c>
       <c r="K9" s="23">
@@ -12761,7 +12831,7 @@
         <v>46286</v>
       </c>
       <c r="E10" s="29">
-        <f>IF($B10&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B10) / 24)</f>
+        <f>IF($B10&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B10) / 24)</f>
         <v>57</v>
       </c>
       <c r="F10" s="15"/>
@@ -12770,12 +12840,12 @@
         <v>16</v>
       </c>
       <c r="H10" s="36">
-        <f>'⚙ Configuración'!$C$10-G10</f>
+        <f>'⚙ Configuración'!$C$11-G10</f>
         <v>60</v>
       </c>
       <c r="I10" s="37"/>
       <c r="J10" s="38">
-        <f>IF($B10&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B10 - 1) / 24)</f>
+        <f>IF($B10&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B10 - 1) / 24)</f>
         <v>19</v>
       </c>
       <c r="K10" s="39"/>
@@ -12793,7 +12863,7 @@
         <v>46289</v>
       </c>
       <c r="E11" s="29">
-        <f>IF($B11&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B11) / 24)</f>
+        <f>IF($B11&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B11) / 24)</f>
         <v>53.833333333333336</v>
       </c>
       <c r="F11" s="15"/>
@@ -12802,12 +12872,12 @@
         <v>16</v>
       </c>
       <c r="H11" s="36">
-        <f>'⚙ Configuración'!$C$10-G11</f>
+        <f>'⚙ Configuración'!$C$11-G11</f>
         <v>60</v>
       </c>
       <c r="I11" s="37"/>
       <c r="J11" s="38">
-        <f>IF($B11&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B11 - 1) / 24)</f>
+        <f>IF($B11&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B11 - 1) / 24)</f>
         <v>22.166666666666668</v>
       </c>
       <c r="K11" s="39"/>
@@ -12825,7 +12895,7 @@
         <v>46293</v>
       </c>
       <c r="E12" s="29">
-        <f>IF($B12&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B12) / 24)</f>
+        <f>IF($B12&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B12) / 24)</f>
         <v>50.666666666666664</v>
       </c>
       <c r="F12" s="15">
@@ -12837,12 +12907,12 @@
         <v>27</v>
       </c>
       <c r="H12" s="36">
-        <f>'⚙ Configuración'!$C$10-G12</f>
+        <f>'⚙ Configuración'!$C$11-G12</f>
         <v>49</v>
       </c>
       <c r="I12" s="37"/>
       <c r="J12" s="38">
-        <f>IF($B12&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B12 - 1) / 24)</f>
+        <f>IF($B12&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B12 - 1) / 24)</f>
         <v>25.333333333333332</v>
       </c>
       <c r="K12" s="39"/>
@@ -12860,7 +12930,7 @@
         <v>46296</v>
       </c>
       <c r="E13" s="29">
-        <f>IF($B13&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B13) / 24)</f>
+        <f>IF($B13&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B13) / 24)</f>
         <v>47.5</v>
       </c>
       <c r="F13" s="15"/>
@@ -12869,12 +12939,12 @@
         <v>27</v>
       </c>
       <c r="H13" s="36">
-        <f>'⚙ Configuración'!$C$10-G13</f>
+        <f>'⚙ Configuración'!$C$11-G13</f>
         <v>49</v>
       </c>
       <c r="I13" s="37"/>
       <c r="J13" s="38">
-        <f>IF($B13&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B13 - 1) / 24)</f>
+        <f>IF($B13&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B13 - 1) / 24)</f>
         <v>28.5</v>
       </c>
       <c r="K13" s="39"/>
@@ -12892,7 +12962,7 @@
         <v>46300</v>
       </c>
       <c r="E14" s="29">
-        <f>IF($B14&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B14) / 24)</f>
+        <f>IF($B14&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B14) / 24)</f>
         <v>44.333333333333336</v>
       </c>
       <c r="F14" s="15">
@@ -12904,12 +12974,12 @@
         <v>35</v>
       </c>
       <c r="H14" s="36">
-        <f>'⚙ Configuración'!$C$10-G14</f>
+        <f>'⚙ Configuración'!$C$11-G14</f>
         <v>41</v>
       </c>
       <c r="I14" s="37"/>
       <c r="J14" s="38">
-        <f>IF($B14&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B14 - 1) / 24)</f>
+        <f>IF($B14&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B14 - 1) / 24)</f>
         <v>31.666666666666668</v>
       </c>
       <c r="K14" s="39"/>
@@ -12927,7 +12997,7 @@
         <v>46303</v>
       </c>
       <c r="E15" s="29">
-        <f>IF($B15&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B15) / 24)</f>
+        <f>IF($B15&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B15) / 24)</f>
         <v>41.166666666666664</v>
       </c>
       <c r="F15" s="15">
@@ -12939,15 +13009,15 @@
         <v>42</v>
       </c>
       <c r="H15" s="36">
-        <f>'⚙ Configuración'!$C$10-G15</f>
+        <f>'⚙ Configuración'!$C$11-G15</f>
         <v>34</v>
       </c>
       <c r="I15" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J15" s="38">
-        <f>IF($B15&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B15 - 1) / 24)</f>
+        <f>IF($B15&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B15 - 1) / 24)</f>
         <v>34.833333333333336</v>
       </c>
       <c r="K15" s="39">
@@ -12970,7 +13040,7 @@
         <v>46307</v>
       </c>
       <c r="E16" s="29">
-        <f>IF($B16&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B16) / 24)</f>
+        <f>IF($B16&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B16) / 24)</f>
         <v>38</v>
       </c>
       <c r="F16" s="15"/>
@@ -12979,12 +13049,12 @@
         <v>42</v>
       </c>
       <c r="H16" s="36">
-        <f>'⚙ Configuración'!$C$10-G16</f>
+        <f>'⚙ Configuración'!$C$11-G16</f>
         <v>34</v>
       </c>
       <c r="I16" s="37"/>
       <c r="J16" s="38">
-        <f>IF($B16&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B16 - 1) / 24)</f>
+        <f>IF($B16&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B16 - 1) / 24)</f>
         <v>38</v>
       </c>
       <c r="K16" s="39"/>
@@ -13001,7 +13071,7 @@
         <v>46310</v>
       </c>
       <c r="E17" s="29">
-        <f>IF($B17&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B17) / 24)</f>
+        <f>IF($B17&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B17) / 24)</f>
         <v>34.833333333333336</v>
       </c>
       <c r="F17" s="15"/>
@@ -13010,12 +13080,12 @@
         <v>42</v>
       </c>
       <c r="H17" s="36">
-        <f>'⚙ Configuración'!$C$10-G17</f>
+        <f>'⚙ Configuración'!$C$11-G17</f>
         <v>34</v>
       </c>
       <c r="I17" s="37"/>
       <c r="J17" s="38">
-        <f>IF($B17&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B17 - 1) / 24)</f>
+        <f>IF($B17&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B17 - 1) / 24)</f>
         <v>41.166666666666664</v>
       </c>
       <c r="K17" s="39"/>
@@ -13032,7 +13102,7 @@
         <v>46314</v>
       </c>
       <c r="E18" s="29">
-        <f>IF($B18&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B18) / 24)</f>
+        <f>IF($B18&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B18) / 24)</f>
         <v>31.666666666666668</v>
       </c>
       <c r="F18" s="15"/>
@@ -13041,12 +13111,12 @@
         <v>42</v>
       </c>
       <c r="H18" s="36">
-        <f>'⚙ Configuración'!$C$10-G18</f>
+        <f>'⚙ Configuración'!$C$11-G18</f>
         <v>34</v>
       </c>
       <c r="I18" s="37"/>
       <c r="J18" s="38">
-        <f>IF($B18&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B18 - 1) / 24)</f>
+        <f>IF($B18&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B18 - 1) / 24)</f>
         <v>44.333333333333336</v>
       </c>
       <c r="K18" s="39"/>
@@ -13063,7 +13133,7 @@
         <v>46317</v>
       </c>
       <c r="E19" s="29">
-        <f>IF($B19&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B19) / 24)</f>
+        <f>IF($B19&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B19) / 24)</f>
         <v>28.5</v>
       </c>
       <c r="F19" s="15"/>
@@ -13072,12 +13142,12 @@
         <v>42</v>
       </c>
       <c r="H19" s="36">
-        <f>'⚙ Configuración'!$C$10-G19</f>
+        <f>'⚙ Configuración'!$C$11-G19</f>
         <v>34</v>
       </c>
       <c r="I19" s="37"/>
       <c r="J19" s="38">
-        <f>IF($B19&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B19 - 1) / 24)</f>
+        <f>IF($B19&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B19 - 1) / 24)</f>
         <v>47.5</v>
       </c>
       <c r="K19" s="39"/>
@@ -13094,7 +13164,7 @@
         <v>46321</v>
       </c>
       <c r="E20" s="29">
-        <f>IF($B20&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B20) / 24)</f>
+        <f>IF($B20&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B20) / 24)</f>
         <v>25.333333333333332</v>
       </c>
       <c r="F20" s="15"/>
@@ -13103,12 +13173,12 @@
         <v>42</v>
       </c>
       <c r="H20" s="36">
-        <f>'⚙ Configuración'!$C$10-G20</f>
+        <f>'⚙ Configuración'!$C$11-G20</f>
         <v>34</v>
       </c>
       <c r="I20" s="37"/>
       <c r="J20" s="38">
-        <f>IF($B20&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B20 - 1) / 24)</f>
+        <f>IF($B20&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B20 - 1) / 24)</f>
         <v>50.666666666666664</v>
       </c>
       <c r="K20" s="39"/>
@@ -13125,7 +13195,7 @@
         <v>46324</v>
       </c>
       <c r="E21" s="29">
-        <f>IF($B21&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B21) / 24)</f>
+        <f>IF($B21&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B21) / 24)</f>
         <v>22.166666666666668</v>
       </c>
       <c r="F21" s="15"/>
@@ -13134,15 +13204,15 @@
         <v>42</v>
       </c>
       <c r="H21" s="36">
-        <f>'⚙ Configuración'!$C$10-G21</f>
+        <f>'⚙ Configuración'!$C$11-G21</f>
         <v>34</v>
       </c>
       <c r="I21" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J21" s="38">
-        <f>IF($B21&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B21 - 1) / 24)</f>
+        <f>IF($B21&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B21 - 1) / 24)</f>
         <v>53.833333333333336</v>
       </c>
       <c r="K21" s="39">
@@ -13164,7 +13234,7 @@
         <v>46328</v>
       </c>
       <c r="E22" s="29">
-        <f>IF($B22&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B22) / 24)</f>
+        <f>IF($B22&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B22) / 24)</f>
         <v>19</v>
       </c>
       <c r="F22" s="15"/>
@@ -13173,12 +13243,12 @@
         <v>42</v>
       </c>
       <c r="H22" s="36">
-        <f>'⚙ Configuración'!$C$10-G22</f>
+        <f>'⚙ Configuración'!$C$11-G22</f>
         <v>34</v>
       </c>
       <c r="I22" s="37"/>
       <c r="J22" s="38">
-        <f>IF($B22&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B22 - 1) / 24)</f>
+        <f>IF($B22&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B22 - 1) / 24)</f>
         <v>57</v>
       </c>
       <c r="K22" s="39"/>
@@ -13195,7 +13265,7 @@
         <v>46331</v>
       </c>
       <c r="E23" s="29">
-        <f>IF($B23&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B23) / 24)</f>
+        <f>IF($B23&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B23) / 24)</f>
         <v>15.833333333333334</v>
       </c>
       <c r="F23" s="15"/>
@@ -13204,12 +13274,12 @@
         <v>42</v>
       </c>
       <c r="H23" s="36">
-        <f>'⚙ Configuración'!$C$10-G23</f>
+        <f>'⚙ Configuración'!$C$11-G23</f>
         <v>34</v>
       </c>
       <c r="I23" s="37"/>
       <c r="J23" s="38">
-        <f>IF($B23&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B23 - 1) / 24)</f>
+        <f>IF($B23&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B23 - 1) / 24)</f>
         <v>60.166666666666664</v>
       </c>
       <c r="K23" s="39"/>
@@ -13226,7 +13296,7 @@
         <v>46335</v>
       </c>
       <c r="E24" s="29">
-        <f>IF($B24&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B24) / 24)</f>
+        <f>IF($B24&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B24) / 24)</f>
         <v>12.666666666666666</v>
       </c>
       <c r="F24" s="15"/>
@@ -13235,12 +13305,12 @@
         <v>42</v>
       </c>
       <c r="H24" s="36">
-        <f>'⚙ Configuración'!$C$10-G24</f>
+        <f>'⚙ Configuración'!$C$11-G24</f>
         <v>34</v>
       </c>
       <c r="I24" s="37"/>
       <c r="J24" s="38">
-        <f>IF($B24&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B24 - 1) / 24)</f>
+        <f>IF($B24&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B24 - 1) / 24)</f>
         <v>63.333333333333336</v>
       </c>
       <c r="K24" s="39"/>
@@ -13257,7 +13327,7 @@
         <v>46338</v>
       </c>
       <c r="E25" s="29">
-        <f>IF($B25&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B25) / 24)</f>
+        <f>IF($B25&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B25) / 24)</f>
         <v>9.5</v>
       </c>
       <c r="F25" s="15"/>
@@ -13266,12 +13336,12 @@
         <v>42</v>
       </c>
       <c r="H25" s="36">
-        <f>'⚙ Configuración'!$C$10-G25</f>
+        <f>'⚙ Configuración'!$C$11-G25</f>
         <v>34</v>
       </c>
       <c r="I25" s="37"/>
       <c r="J25" s="38">
-        <f>IF($B25&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B25 - 1) / 24)</f>
+        <f>IF($B25&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B25 - 1) / 24)</f>
         <v>66.5</v>
       </c>
       <c r="K25" s="39"/>
@@ -13288,7 +13358,7 @@
         <v>46335</v>
       </c>
       <c r="E26" s="29">
-        <f>IF($B26&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B26) / 24)</f>
+        <f>IF($B26&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B26) / 24)</f>
         <v>6.333333333333333</v>
       </c>
       <c r="F26" s="15"/>
@@ -13297,12 +13367,12 @@
         <v>42</v>
       </c>
       <c r="H26" s="36">
-        <f>'⚙ Configuración'!$C$10-G26</f>
+        <f>'⚙ Configuración'!$C$11-G26</f>
         <v>34</v>
       </c>
       <c r="I26" s="37"/>
       <c r="J26" s="38">
-        <f>IF($B26&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B26 - 1) / 24)</f>
+        <f>IF($B26&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B26 - 1) / 24)</f>
         <v>69.666666666666671</v>
       </c>
       <c r="K26" s="39"/>
@@ -13319,7 +13389,7 @@
         <v>46342</v>
       </c>
       <c r="E27" s="29">
-        <f>IF($B27&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B27) / 24)</f>
+        <f>IF($B27&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B27) / 24)</f>
         <v>3.1666666666666665</v>
       </c>
       <c r="F27" s="15"/>
@@ -13328,12 +13398,12 @@
         <v>42</v>
       </c>
       <c r="H27" s="36">
-        <f>'⚙ Configuración'!$C$10-G27</f>
+        <f>'⚙ Configuración'!$C$11-G27</f>
         <v>34</v>
       </c>
       <c r="I27" s="37"/>
       <c r="J27" s="38">
-        <f>IF($B27&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B27 - 1) / 24)</f>
+        <f>IF($B27&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B27 - 1) / 24)</f>
         <v>72.833333333333329</v>
       </c>
       <c r="K27" s="39"/>
@@ -13350,7 +13420,7 @@
         <v>46345</v>
       </c>
       <c r="E28" s="29">
-        <f>IF($B28&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B28) / 24)</f>
+        <f>IF($B28&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B28) / 24)</f>
         <v>0</v>
       </c>
       <c r="F28" s="15"/>
@@ -13359,19 +13429,19 @@
         <v>42</v>
       </c>
       <c r="H28" s="36">
-        <f>'⚙ Configuración'!$C$10-G28</f>
+        <f>'⚙ Configuración'!$C$11-G28</f>
         <v>34</v>
       </c>
       <c r="I28" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J28" s="38">
-        <f>IF($B28&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B28 - 1) / 24)</f>
+        <f>IF($B28&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B28 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K28" s="39">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="L28" s="39">
@@ -13389,7 +13459,7 @@
         <v>46349</v>
       </c>
       <c r="E29" s="29">
-        <f>IF($B29&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B29) / 24)</f>
+        <f>IF($B29&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B29) / 24)</f>
         <v>0</v>
       </c>
       <c r="F29" s="15"/>
@@ -13398,12 +13468,12 @@
         <v>42</v>
       </c>
       <c r="H29" s="36">
-        <f>'⚙ Configuración'!$C$10-G29</f>
+        <f>'⚙ Configuración'!$C$11-G29</f>
         <v>34</v>
       </c>
       <c r="I29" s="37"/>
       <c r="J29" s="38">
-        <f>IF($B29&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B29 - 1) / 24)</f>
+        <f>IF($B29&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B29 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K29" s="39"/>
@@ -13420,7 +13490,7 @@
         <v>46352</v>
       </c>
       <c r="E30" s="29">
-        <f>IF($B30&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B30) / 24)</f>
+        <f>IF($B30&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B30) / 24)</f>
         <v>0</v>
       </c>
       <c r="F30" s="15"/>
@@ -13429,12 +13499,12 @@
         <v>42</v>
       </c>
       <c r="H30" s="36">
-        <f>'⚙ Configuración'!$C$10-G30</f>
+        <f>'⚙ Configuración'!$C$11-G30</f>
         <v>34</v>
       </c>
       <c r="I30" s="37"/>
       <c r="J30" s="38">
-        <f>IF($B30&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B30 - 1) / 24)</f>
+        <f>IF($B30&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B30 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K30" s="39"/>
@@ -13451,7 +13521,7 @@
         <v>46356</v>
       </c>
       <c r="E31" s="29">
-        <f>IF($B31&gt;=25, 0, '⚙ Configuración'!$C$10 * (25 - $B31) / 24)</f>
+        <f>IF($B31&gt;=25, 0, '⚙ Configuración'!$C$11 * (25 - $B31) / 24)</f>
         <v>0</v>
       </c>
       <c r="F31" s="15"/>
@@ -13460,15 +13530,15 @@
         <v>42</v>
       </c>
       <c r="H31" s="36">
-        <f>'⚙ Configuración'!$C$10-G31</f>
+        <f>'⚙ Configuración'!$C$11-G31</f>
         <v>34</v>
       </c>
       <c r="I31" s="37">
-        <f>'⚙ Configuración'!$C$10</f>
+        <f>'⚙ Configuración'!$C$11</f>
         <v>76</v>
       </c>
       <c r="J31" s="38">
-        <f>IF($B31&gt;=25, '⚙ Configuración'!$C$10, '⚙ Configuración'!$C$10 * ($B31 - 1) / 24)</f>
+        <f>IF($B31&gt;=25, '⚙ Configuración'!$C$11, '⚙ Configuración'!$C$11 * ($B31 - 1) / 24)</f>
         <v>76</v>
       </c>
       <c r="K31" s="39"/>
@@ -13482,31 +13552,69 @@
       <c r="E33" s="55"/>
     </row>
     <row r="34" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="23"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
+      <c r="B34" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="C34" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>179</v>
+      </c>
       <c r="E34" s="23"/>
     </row>
     <row r="35" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="23"/>
-      <c r="C35" s="23"/>
-      <c r="D35" s="23"/>
+      <c r="B35" s="23">
+        <v>1</v>
+      </c>
+      <c r="C35" s="23">
+        <v>13</v>
+      </c>
+      <c r="D35" s="23">
+        <f>C35</f>
+        <v>13</v>
+      </c>
       <c r="E35" s="23"/>
     </row>
     <row r="36" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="23"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="23"/>
+      <c r="B36" s="23">
+        <v>2</v>
+      </c>
+      <c r="C36" s="23">
+        <v>29</v>
+      </c>
+      <c r="D36" s="23">
+        <f>C36+D35</f>
+        <v>42</v>
+      </c>
       <c r="E36" s="23"/>
     </row>
     <row r="37" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="23"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="23"/>
+      <c r="B37" s="23">
+        <v>3</v>
+      </c>
+      <c r="C37" s="23">
+        <v>21</v>
+      </c>
+      <c r="D37" s="23">
+        <f t="shared" ref="D37:D38" si="1">C37+D36</f>
+        <v>63</v>
+      </c>
       <c r="E37" s="23"/>
       <c r="H37" s="67"/>
     </row>
-    <row r="38" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="71">
+        <v>4</v>
+      </c>
+      <c r="C38" s="71">
+        <v>13</v>
+      </c>
+      <c r="D38" s="23">
+        <f t="shared" si="1"/>
+        <v>76</v>
+      </c>
+    </row>
     <row r="39" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -14499,28 +14607,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="79" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="73"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="76"/>
     </row>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="73"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="81" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72"/>
-      <c r="E3" s="73"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="76"/>
     </row>
     <row r="4" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="41" t="s">
@@ -14601,12 +14709,12 @@
       <c r="E9" s="45"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="82" t="s">
         <v>118</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="73"/>
+      <c r="C10" s="75"/>
+      <c r="D10" s="75"/>
+      <c r="E10" s="76"/>
     </row>
     <row r="11" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
@@ -14625,7 +14733,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="42">
-        <f>'⚙ Configuración'!C11</f>
+        <f>'⚙ Configuración'!C12</f>
         <v>16</v>
       </c>
       <c r="D12" s="43" t="s">
@@ -14638,7 +14746,7 @@
         <v>122</v>
       </c>
       <c r="C13" s="47">
-        <f>C11-'⚙ Configuración'!C11</f>
+        <f>C11-'⚙ Configuración'!C12</f>
         <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -14651,7 +14759,7 @@
         <v>124</v>
       </c>
       <c r="C14" s="48">
-        <f>IFERROR(C11/'⚙ Configuración'!C12,0)</f>
+        <f>IFERROR(C11/'⚙ Configuración'!C13,0)</f>
         <v>5.2</v>
       </c>
       <c r="D14" s="43" t="s">
@@ -14664,7 +14772,7 @@
         <v>126</v>
       </c>
       <c r="C15" s="49">
-        <f>IFERROR(C11/('⚙ Configuración'!C12*'⚙ Configuración'!C9),0)</f>
+        <f>IFERROR(C11/('⚙ Configuración'!C13*'⚙ Configuración'!C9),0)</f>
         <v>0.8666666666666667</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -14673,12 +14781,12 @@
       <c r="E15" s="45"/>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="91" t="s">
+      <c r="B16" s="83" t="s">
         <v>128</v>
       </c>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="73"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="76"/>
     </row>
     <row r="17" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
@@ -14722,8 +14830,8 @@
         <v>135</v>
       </c>
       <c r="C20" s="48">
-        <f>IF(C17=0,0,'📋 Sprint Backlog'!G28/C17)</f>
-        <v>7</v>
+        <f>IF(C17=0,0,'⚙ Configuración'!C10/C17)</f>
+        <v>4.833333333333333</v>
       </c>
       <c r="D20" s="43" t="s">
         <v>136</v>
@@ -14736,7 +14844,7 @@
       </c>
       <c r="C21" s="49">
         <f>IF(C17=0,1,C20/IFERROR(('⚙ Configuración'!C10/'⚙ Configuración'!C9),1))</f>
-        <v>0.55263157894736847</v>
+        <v>1</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>138</v>
@@ -14744,52 +14852,52 @@
       <c r="E21" s="45"/>
     </row>
     <row r="22" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="92" t="s">
+      <c r="B22" s="84" t="s">
         <v>139</v>
       </c>
-      <c r="C22" s="72"/>
-      <c r="D22" s="72"/>
-      <c r="E22" s="73"/>
+      <c r="C22" s="75"/>
+      <c r="D22" s="75"/>
+      <c r="E22" s="76"/>
     </row>
     <row r="23" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="51" t="s">
         <v>140</v>
       </c>
-      <c r="C23" s="93" t="s">
+      <c r="C23" s="85" t="s">
         <v>141</v>
       </c>
-      <c r="D23" s="72"/>
-      <c r="E23" s="73"/>
+      <c r="D23" s="75"/>
+      <c r="E23" s="76"/>
     </row>
     <row r="24" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="52" t="s">
         <v>142</v>
       </c>
-      <c r="C24" s="88" t="s">
+      <c r="C24" s="74" t="s">
         <v>143</v>
       </c>
-      <c r="D24" s="72"/>
-      <c r="E24" s="73"/>
+      <c r="D24" s="75"/>
+      <c r="E24" s="76"/>
     </row>
     <row r="25" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="53" t="s">
         <v>144</v>
       </c>
-      <c r="C25" s="89" t="s">
+      <c r="C25" s="77" t="s">
         <v>145</v>
       </c>
-      <c r="D25" s="72"/>
-      <c r="E25" s="73"/>
+      <c r="D25" s="75"/>
+      <c r="E25" s="76"/>
     </row>
     <row r="26" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="C26" s="90" t="s">
+      <c r="C26" s="78" t="s">
         <v>147</v>
       </c>
-      <c r="D26" s="72"/>
-      <c r="E26" s="73"/>
+      <c r="D26" s="75"/>
+      <c r="E26" s="76"/>
     </row>
     <row r="27" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15797,103 +15905,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="C1" s="71" t="s">
+      <c r="C1" s="79" t="s">
         <v>148</v>
       </c>
-      <c r="D1" s="72"/>
-      <c r="E1" s="73"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="76"/>
     </row>
     <row r="2" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C2" s="96" t="s">
+      <c r="C2" s="99" t="s">
         <v>172</v>
       </c>
-      <c r="D2" s="72"/>
-      <c r="E2" s="73"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
     </row>
     <row r="3" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C3" s="97" t="s">
+      <c r="C3" s="100" t="s">
         <v>149</v>
       </c>
-      <c r="D3" s="72"/>
-      <c r="E3" s="73"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="76"/>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C4" s="93" t="s">
+      <c r="C4" s="85" t="s">
         <v>150</v>
       </c>
-      <c r="D4" s="72"/>
-      <c r="E4" s="73"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="76"/>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C5" s="93" t="s">
+      <c r="C5" s="85" t="s">
         <v>176</v>
       </c>
-      <c r="D5" s="72"/>
-      <c r="E5" s="73"/>
+      <c r="D5" s="75"/>
+      <c r="E5" s="76"/>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C6" s="93"/>
-      <c r="D6" s="72"/>
-      <c r="E6" s="73"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="75"/>
+      <c r="E6" s="76"/>
     </row>
     <row r="8" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C8" s="98" t="s">
+      <c r="C8" s="101" t="s">
         <v>151</v>
       </c>
-      <c r="D8" s="72"/>
-      <c r="E8" s="73"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="76"/>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C9" s="99" t="s">
+      <c r="C9" s="102" t="s">
         <v>173</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="73"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="76"/>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C10" s="99" t="s">
+      <c r="C10" s="102" t="s">
         <v>175</v>
       </c>
-      <c r="D10" s="72"/>
-      <c r="E10" s="73"/>
+      <c r="D10" s="75"/>
+      <c r="E10" s="76"/>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C11" s="90"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="73"/>
+      <c r="C11" s="78"/>
+      <c r="D11" s="75"/>
+      <c r="E11" s="76"/>
     </row>
     <row r="13" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C13" s="100" t="s">
+      <c r="C13" s="103" t="s">
         <v>152</v>
       </c>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="D13" s="75"/>
+      <c r="E13" s="76"/>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C14" s="94" t="s">
+      <c r="C14" s="97" t="s">
         <v>177</v>
       </c>
-      <c r="D14" s="72"/>
-      <c r="E14" s="73"/>
+      <c r="D14" s="75"/>
+      <c r="E14" s="76"/>
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C15" s="94" t="s">
+      <c r="C15" s="97" t="s">
         <v>174</v>
       </c>
-      <c r="D15" s="72"/>
-      <c r="E15" s="73"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="76"/>
     </row>
     <row r="16" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C16" s="88"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="73"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="76"/>
     </row>
     <row r="18" spans="3:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C18" s="95" t="s">
+      <c r="C18" s="98" t="s">
         <v>153</v>
       </c>
-      <c r="D18" s="72"/>
-      <c r="E18" s="73"/>
+      <c r="D18" s="75"/>
+      <c r="E18" s="76"/>
     </row>
     <row r="19" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C19" s="56" t="s">

</xml_diff>